<commit_message>
feat(projections): add FISV tab to projections workbook
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -8,6 +8,7 @@
     <sheet name="ELF" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="SOFI" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="CRM" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FISV" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12313,4 +12314,2369 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>FISV</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46193</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>530</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>21500</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>4850</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>5460</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>6100</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>17</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>19</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>530</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>21500</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>4850</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>5460</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>6100</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>13</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>13</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>13</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>530</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>21500</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>4850</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>5460</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>6100</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(projections): add ZETA tab to projections workbook
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -9,6 +9,7 @@
     <sheet name="SOFI" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="CRM" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="FISV" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ZETA" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14679,4 +14680,2369 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>ZETA</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>1785</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.204</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.233</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.264</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>238</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>238</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>298</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>343</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>400</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.213</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>250</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>1785</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.224</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>238</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>238</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>298</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>343</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>400</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.173</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.186</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>250</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>1785</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.143</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.127</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.152</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>238</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>238</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>298</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>343</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>400</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.124</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.131</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.138</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>12</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>12</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>12</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>12</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>12</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(projections): add HOOD tab to projections workbook
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -10,6 +10,7 @@
     <sheet name="CRM" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="FISV" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="ZETA" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="HOOD" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17045,4 +17046,2369 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>915</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>5100</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>42</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>42</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>42</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>42</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>42</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>915</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>5100</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>25</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>25</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>25</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>25</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>25</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>33</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>33</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>33</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>33</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>33</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>915</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>5100</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(projections): add NFLX tab to projections workbook
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -11,6 +11,7 @@
     <sheet name="FISV" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="ZETA" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="HOOD" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="NFLX" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19411,4 +19412,2369 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>4300</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>51200</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>13300</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>13300</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>15300</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>17600</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>20200</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>38</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>38</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>38</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>38</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>38</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>4300</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>51200</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>13300</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>13300</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>15300</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>17600</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>20200</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>24</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>24</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>24</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>24</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>24</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>4300</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>51200</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>13300</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>13300</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>15300</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>17600</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>20200</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>18</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>18</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>18</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>18</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>18</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>24</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>24</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>24</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>24</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>24</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(projections): add NOW (ServiceNow) tab to projections workbook
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -12,6 +12,7 @@
     <sheet name="ZETA" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="HOOD" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="NFLX" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="NOW" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1783,6 +1784,2371 @@
       </c>
       <c r="H67" s="84" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>1050</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>16200</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>5300</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>6300</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>7400</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>28</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>28</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>28</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>28</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>28</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>35</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>35</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>35</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>35</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>35</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>1050</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>16200</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>5300</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>6300</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>7400</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>28</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>28</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>28</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>28</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>28</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>1050</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>16200</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>5300</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>6300</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>7400</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="68" ht="16.5" customHeight="1" s="92">

</xml_diff>

<commit_message>
feat(projections): add QXO tab to projections workbook
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -13,6 +13,7 @@
     <sheet name="HOOD" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="NFLX" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="NOW" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="QXO" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5225,6 +5226,2371 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>QXO</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>800</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>13000</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>450</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>450</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>780</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>1150</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>40</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>40</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>40</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>40</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>40</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>800</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>13000</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>450</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>450</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>780</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>1150</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>800</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>13000</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>450</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>450</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>780</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>1150</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(projections): add CEG (Constellation Energy) tab to projections workbook
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -14,6 +14,7 @@
     <sheet name="NFLX" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="NOW" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="QXO" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="CEG" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7591,6 +7592,2371 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>34500</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>4150</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>4227</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>4892</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>5630</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>6460</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>26</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>26</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>26</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>26</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>26</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>34</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>34</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>34</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>34</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>34</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>361</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>34500</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>4150</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>4227</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>4892</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>5630</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>6460</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.136</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.151</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>28</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>28</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>28</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>28</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>28</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>361</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>34500</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>4150</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>4227</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>4892</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>5630</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>6460</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.135</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>16</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>22</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(projections): add UBER (Uber Technologies) tab to projections workbook
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -15,6 +15,7 @@
     <sheet name="NOW" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="QXO" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="CEG" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="UBER" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9957,6 +9958,2371 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>UBER</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>2080</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>59500</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>8900</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>11200</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>13700</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>32</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>2080</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>59500</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>8900</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>11200</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>13700</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.155</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>20</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>26</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>26</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>26</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>26</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>26</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>2080</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>59500</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>8900</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>11200</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>13700</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>20</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>20</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>20</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>20</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>20</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(projections): add ORCL tab to projections workbook
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -16,6 +16,7 @@
     <sheet name="QXO" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="CEG" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="UBER" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="ORCL" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12323,6 +12324,2371 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>2910</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>67357</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>22200</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>22200</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>23300</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>28200</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>33500</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>28</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>28</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>28</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>28</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>28</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>38</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>38</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>38</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>38</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>38</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>2910</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>67357</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>22200</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>22200</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>23300</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>28200</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>33500</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>30</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>2910</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>67357</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>22200</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>22200</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>23300</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>28200</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>33500</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>20</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>20</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>20</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>20</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>20</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(projections): add BABA tab to projections workbook
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -17,6 +17,7 @@
     <sheet name="CEG" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="UBER" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="ORCL" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="BABA" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14689,6 +14690,2371 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>BABA</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>148401</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>15400</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>15400</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>18000</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>21000</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>24000</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>22</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>22</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>22</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>22</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>22</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>148401</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>15400</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>15400</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>18000</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>21000</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>24000</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>18</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>18</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>18</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>18</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>18</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>148401</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>15400</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>15400</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>18000</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>21000</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>24000</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>8</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>8</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>8</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>8</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>8</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>12</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>12</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>12</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>12</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>12</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(projections): add NU tab to projections workbook
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -18,6 +18,7 @@
     <sheet name="UBER" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="ORCL" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="BABA" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="NU" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17055,6 +17056,2371 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>NU</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>4900</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>21000</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>3800</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>3800</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>4900</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>6200</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>7700</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>4900</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>21000</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>3800</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>3800</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>4900</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>6200</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>7700</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>14</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>14</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>14</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>14</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>14</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>4900</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>21000</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>3800</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>3800</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>4900</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>6200</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>7700</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>14</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(projections): add PLTR tab to projections workbook
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -19,6 +19,7 @@
     <sheet name="ORCL" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="BABA" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="NU" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="PLTR" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19421,6 +19422,2371 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>2570</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>7716</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>3449</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>3449</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>4829</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>7307</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>9500</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>150</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>150</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>150</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>150</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>150</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>2570</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>7716</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>3449</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>3449</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>4829</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>7307</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>9500</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>70</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>70</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>70</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>70</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>70</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>110</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>110</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>110</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>110</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>110</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>2570</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>7716</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>3449</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>3449</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>4829</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>7307</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>9500</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>40</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>40</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>40</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>40</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>40</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>65</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>65</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>65</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>65</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>65</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
fix(projections): compress PLTR PE multiples over time as growth decelerates
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -19738,22 +19738,22 @@
         </is>
       </c>
       <c r="C18" s="25" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E18" s="25" t="n">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="F18" s="25" t="n">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>100</v>
+        <v>52</v>
       </c>
       <c r="H18" s="26" t="n">
-        <v>100</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="92">
@@ -19763,22 +19763,22 @@
         </is>
       </c>
       <c r="C19" s="25" t="n">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="E19" s="25" t="n">
-        <v>150</v>
+        <v>110</v>
       </c>
       <c r="F19" s="25" t="n">
-        <v>150</v>
+        <v>88</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>150</v>
+        <v>72</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>150</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="92">
@@ -20204,22 +20204,22 @@
         </is>
       </c>
       <c r="C42" s="55" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D42" s="55" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E42" s="55" t="n">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="F42" s="55" t="n">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="G42" s="55" t="n">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="H42" s="56" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" s="92">
@@ -20229,22 +20229,22 @@
         </is>
       </c>
       <c r="C43" s="55" t="n">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D43" s="55" t="n">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="E43" s="55" t="n">
-        <v>110</v>
+        <v>75</v>
       </c>
       <c r="F43" s="55" t="n">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="G43" s="55" t="n">
-        <v>110</v>
+        <v>50</v>
       </c>
       <c r="H43" s="56" t="n">
-        <v>110</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" s="92">
@@ -20670,22 +20670,22 @@
         </is>
       </c>
       <c r="C66" s="83" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="D66" s="83" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E66" s="83" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="F66" s="83" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G66" s="83" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="H66" s="84" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
     </row>
     <row r="67" ht="16.5" customHeight="1" s="92">
@@ -20695,22 +20695,22 @@
         </is>
       </c>
       <c r="C67" s="83" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="D67" s="83" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E67" s="83" t="n">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="F67" s="83" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="G67" s="83" t="n">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="H67" s="84" t="n">
-        <v>65</v>
+        <v>26</v>
       </c>
     </row>
     <row r="68" ht="16.5" customHeight="1" s="92">

</xml_diff>

<commit_message>
fix(projections): compress PE multiples over time for high-deceleration tabs (QXO, ORCL, NOW, NU, ZETA)
Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -3183,22 +3183,22 @@
         </is>
       </c>
       <c r="C18" s="25" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E18" s="25" t="n">
         <v>28</v>
       </c>
       <c r="F18" s="25" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H18" s="26" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="92">
@@ -3208,22 +3208,22 @@
         </is>
       </c>
       <c r="C19" s="25" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E19" s="25" t="n">
         <v>35</v>
       </c>
       <c r="F19" s="25" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="92">
@@ -3649,22 +3649,22 @@
         </is>
       </c>
       <c r="C42" s="55" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D42" s="55" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E42" s="55" t="n">
         <v>22</v>
       </c>
       <c r="F42" s="55" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G42" s="55" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H42" s="56" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" s="92">
@@ -3674,22 +3674,22 @@
         </is>
       </c>
       <c r="C43" s="55" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D43" s="55" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E43" s="55" t="n">
         <v>28</v>
       </c>
       <c r="F43" s="55" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G43" s="55" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H43" s="56" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" s="92">
@@ -4115,22 +4115,22 @@
         </is>
       </c>
       <c r="C66" s="83" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D66" s="83" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E66" s="83" t="n">
         <v>16</v>
       </c>
       <c r="F66" s="83" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G66" s="83" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H66" s="84" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="67" ht="16.5" customHeight="1" s="92">
@@ -4140,22 +4140,22 @@
         </is>
       </c>
       <c r="C67" s="83" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D67" s="83" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E67" s="83" t="n">
         <v>22</v>
       </c>
       <c r="F67" s="83" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G67" s="83" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H67" s="84" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="68" ht="16.5" customHeight="1" s="92">
@@ -5548,22 +5548,22 @@
         </is>
       </c>
       <c r="C18" s="25" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D18" s="25" t="n">
         <v>30</v>
       </c>
       <c r="E18" s="25" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F18" s="25" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="H18" s="26" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="92">
@@ -5573,22 +5573,22 @@
         </is>
       </c>
       <c r="C19" s="25" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D19" s="25" t="n">
         <v>40</v>
       </c>
       <c r="E19" s="25" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F19" s="25" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="92">
@@ -6014,22 +6014,22 @@
         </is>
       </c>
       <c r="C42" s="55" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D42" s="55" t="n">
         <v>22</v>
       </c>
       <c r="E42" s="55" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F42" s="55" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G42" s="55" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="H42" s="56" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" s="92">
@@ -6039,22 +6039,22 @@
         </is>
       </c>
       <c r="C43" s="55" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D43" s="55" t="n">
         <v>30</v>
       </c>
       <c r="E43" s="55" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F43" s="55" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G43" s="55" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H43" s="56" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" s="92">
@@ -6480,22 +6480,22 @@
         </is>
       </c>
       <c r="C66" s="83" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D66" s="83" t="n">
         <v>14</v>
       </c>
       <c r="E66" s="83" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F66" s="83" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G66" s="83" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H66" s="84" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="67" ht="16.5" customHeight="1" s="92">
@@ -6505,22 +6505,22 @@
         </is>
       </c>
       <c r="C67" s="83" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D67" s="83" t="n">
         <v>22</v>
       </c>
       <c r="E67" s="83" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F67" s="83" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G67" s="83" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H67" s="84" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="68" ht="16.5" customHeight="1" s="92">
@@ -12643,22 +12643,22 @@
         </is>
       </c>
       <c r="C18" s="25" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E18" s="25" t="n">
         <v>28</v>
       </c>
       <c r="F18" s="25" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="H18" s="26" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="92">
@@ -12668,22 +12668,22 @@
         </is>
       </c>
       <c r="C19" s="25" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E19" s="25" t="n">
         <v>38</v>
       </c>
       <c r="F19" s="25" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>38</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="92">
@@ -13109,22 +13109,22 @@
         </is>
       </c>
       <c r="C42" s="55" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D42" s="55" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E42" s="55" t="n">
         <v>22</v>
       </c>
       <c r="F42" s="55" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G42" s="55" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H42" s="56" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" s="92">
@@ -13134,22 +13134,22 @@
         </is>
       </c>
       <c r="C43" s="55" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D43" s="55" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E43" s="55" t="n">
         <v>30</v>
       </c>
       <c r="F43" s="55" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G43" s="55" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="H43" s="56" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" s="92">
@@ -13575,22 +13575,22 @@
         </is>
       </c>
       <c r="C66" s="83" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D66" s="83" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E66" s="83" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F66" s="83" t="n">
         <v>14</v>
       </c>
       <c r="G66" s="83" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H66" s="84" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="67" ht="16.5" customHeight="1" s="92">
@@ -13600,22 +13600,22 @@
         </is>
       </c>
       <c r="C67" s="83" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D67" s="83" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E67" s="83" t="n">
         <v>20</v>
       </c>
       <c r="F67" s="83" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G67" s="83" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H67" s="84" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="68" ht="16.5" customHeight="1" s="92">
@@ -17373,22 +17373,22 @@
         </is>
       </c>
       <c r="C18" s="25" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E18" s="25" t="n">
         <v>20</v>
       </c>
       <c r="F18" s="25" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H18" s="26" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="92">
@@ -17398,22 +17398,22 @@
         </is>
       </c>
       <c r="C19" s="25" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D19" s="25" t="n">
         <v>30</v>
       </c>
       <c r="E19" s="25" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F19" s="25" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="92">
@@ -17839,22 +17839,22 @@
         </is>
       </c>
       <c r="C42" s="55" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D42" s="55" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E42" s="55" t="n">
         <v>14</v>
       </c>
       <c r="F42" s="55" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G42" s="55" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H42" s="56" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" s="92">
@@ -17864,22 +17864,22 @@
         </is>
       </c>
       <c r="C43" s="55" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D43" s="55" t="n">
         <v>22</v>
       </c>
       <c r="E43" s="55" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F43" s="55" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G43" s="55" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="H43" s="56" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" s="92">
@@ -18305,10 +18305,10 @@
         </is>
       </c>
       <c r="C66" s="83" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D66" s="83" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E66" s="83" t="n">
         <v>9</v>
@@ -18317,10 +18317,10 @@
         <v>9</v>
       </c>
       <c r="G66" s="83" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H66" s="84" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="67" ht="16.5" customHeight="1" s="92">
@@ -18330,22 +18330,22 @@
         </is>
       </c>
       <c r="C67" s="83" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D67" s="83" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E67" s="83" t="n">
         <v>14</v>
       </c>
       <c r="F67" s="83" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G67" s="83" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H67" s="84" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="68" ht="16.5" customHeight="1" s="92">
@@ -33928,10 +33928,10 @@
         </is>
       </c>
       <c r="C18" s="25" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E18" s="25" t="n">
         <v>18</v>
@@ -33940,10 +33940,10 @@
         <v>18</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H18" s="26" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="92">
@@ -33953,22 +33953,22 @@
         </is>
       </c>
       <c r="C19" s="25" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E19" s="25" t="n">
         <v>24</v>
       </c>
       <c r="F19" s="25" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="92">
@@ -34394,10 +34394,10 @@
         </is>
       </c>
       <c r="C42" s="55" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D42" s="55" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E42" s="55" t="n">
         <v>15</v>
@@ -34406,10 +34406,10 @@
         <v>15</v>
       </c>
       <c r="G42" s="55" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H42" s="56" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" s="92">
@@ -34419,22 +34419,22 @@
         </is>
       </c>
       <c r="C43" s="55" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D43" s="55" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E43" s="55" t="n">
         <v>20</v>
       </c>
       <c r="F43" s="55" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G43" s="55" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H43" s="56" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" s="92">
@@ -34860,10 +34860,10 @@
         </is>
       </c>
       <c r="C66" s="83" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D66" s="83" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E66" s="83" t="n">
         <v>12</v>
@@ -34872,10 +34872,10 @@
         <v>12</v>
       </c>
       <c r="G66" s="83" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H66" s="84" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="67" ht="16.5" customHeight="1" s="92">
@@ -34885,10 +34885,10 @@
         </is>
       </c>
       <c r="C67" s="83" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D67" s="83" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E67" s="83" t="n">
         <v>16</v>
@@ -34897,10 +34897,10 @@
         <v>16</v>
       </c>
       <c r="G67" s="83" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H67" s="84" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="68" ht="16.5" customHeight="1" s="92">

</xml_diff>

<commit_message>
Add INTR (Inter & Co) projection tab
Clone PLTR tab and update for Inter & Co (NASDAQ: INTR), a Brazilian
digital bank. USD-per-share basis (IFRS NI translated ~5.5 BRL/USD).

- ~442M shares; FY2026E rev ~$1.45B, NI ~$335M (~23% margin), EPS ~$0.76
- Analyst FY26-29 NI $335/430/540/650M (EPS $0.76/0.97/1.22/1.47)
- Low bank multiples (8-18x) compressing as growth decelerates
- Base yr-1 $8.3-11.4 (~$9.38 avg PT); bear $6.1-8.3; bull to $13.6

Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -20,6 +20,7 @@
     <sheet name="BABA" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="NU" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="PLTR" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="INTR" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21787,6 +21788,2371 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>INTR</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>442</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>1450</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>335</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>335</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>430</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>540</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>650</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.255</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.28</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>11</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>17</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>15</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>442</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>1450</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>335</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>335</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>430</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>540</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>650</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.255</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>11</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>9</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>8</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>14</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>13</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>12</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>11</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>442</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>1450</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>335</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>335</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>430</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>540</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>650</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.225</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>8</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>8</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>6</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>11</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>10</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>10</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>8</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
INTR: lift and flatten P/E multiples
INTR is cheap/undervalued, so multiples shouldn't compress over time.
- Bull: flat 15-20x (was compressing 13->10 / 18->13)
- Base: flat 13-17x (was compressing 11->8 / 15->11)
- Bear: flat 10-13x, less pessimistic (was 8->6 / 11->8)

Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -22104,22 +22104,22 @@
         </is>
       </c>
       <c r="C18" s="25" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E18" s="25" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F18" s="25" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G18" s="25" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H18" s="26" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="92">
@@ -22129,22 +22129,22 @@
         </is>
       </c>
       <c r="C19" s="25" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D19" s="25" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E19" s="25" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F19" s="25" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G19" s="25" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H19" s="26" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="92">
@@ -22570,22 +22570,22 @@
         </is>
       </c>
       <c r="C42" s="55" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D42" s="55" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E42" s="55" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F42" s="55" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G42" s="55" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="H42" s="56" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" s="92">
@@ -22595,22 +22595,22 @@
         </is>
       </c>
       <c r="C43" s="55" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D43" s="55" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E43" s="55" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F43" s="55" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G43" s="55" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H43" s="56" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" s="92">
@@ -23036,22 +23036,22 @@
         </is>
       </c>
       <c r="C66" s="83" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D66" s="83" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E66" s="83" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F66" s="83" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G66" s="83" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H66" s="84" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="67" ht="16.5" customHeight="1" s="92">
@@ -23061,22 +23061,22 @@
         </is>
       </c>
       <c r="C67" s="83" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D67" s="83" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E67" s="83" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F67" s="83" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G67" s="83" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="H67" s="84" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="68" ht="16.5" customHeight="1" s="92">

</xml_diff>

<commit_message>
Add FOUR (Shift4 Payments) projection tab
Clone INTR tab and update for Shift4 Payments (NYSE: FOUR), a US
integrated-payments company. Non-GAAP basis; revenue line = GRLNF
(gross revenue less network fees), the metric mgmt guides on.

- ~95M fully-diluted economic shares
- FY2026E GRLNF $2,550M (guide $2.5-2.6B), non-GAAP NI ~$532M (EPS ~$5.60)
- Analyst FY26-29 NI $532/656/789/931M (EPS $5.60/6.91/8.31/9.80)
- Payments multiples 7-21x, mild compression; floors kept reasonable (stock ~7x fwd)
- Bear yr-1 $39-50 (~current ~$40.65 / $50 low PT); base $62-84 (~$64 avg PT); bull to ~$118

Amp-Thread-ID: https://ampcode.com/threads/T-019ee60a-8609-761e-9ca7-ea593414dffe
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/projections/Projections.xlsx
+++ b/projections/Projections.xlsx
@@ -21,6 +21,7 @@
     <sheet name="NU" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="PLTR" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="INTR" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="FOUR" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24153,6 +24154,2371 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:J73"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="10.88" customWidth="1" style="92" min="1" max="1"/>
+    <col width="14.38" customWidth="1" style="92" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.5" customHeight="1" s="92"/>
+    <row r="2" ht="16.5" customHeight="1" s="92">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>FOUR</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="92"/>
+    <row r="4" ht="16.5" customHeight="1" s="92">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Bull Case</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="92">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="92">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D6" s="11">
+        <f>(C6*C7) + C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>(D6*D7) + D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>(E6*E7) + E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>(F6*F7) + F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>(G6*G7) + G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="92">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="92">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="26" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="92">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>532</v>
+      </c>
+      <c r="D9" s="19">
+        <f>D6*D14</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>E6*E14</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>F6*F14</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>G6*G14</f>
+        <v/>
+      </c>
+      <c r="H9" s="20">
+        <f>H6*H14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="92">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D10" s="21">
+        <f>(D9-C9)/C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>(E9-D9)/D9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>(F9-E9)/E9</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>(G9-F9)/F9</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>(H9-G9)/G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" s="92">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1" s="92">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>532</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>656</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>789</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>931</v>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1" s="92">
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="26" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" s="92">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>C9/C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="92">
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="26" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="92">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="23">
+        <f>C9/H4</f>
+        <v/>
+      </c>
+      <c r="D16" s="23">
+        <f>D9/H4</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>E9/H4</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>F9/H4</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>G9/H4</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>H9/H4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="92">
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="92">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>15</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>15</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="H18" s="26" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="92">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>21</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>19</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="92">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="26" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="92">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>C18*C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D18*D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="19">
+        <f>E18*E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="19">
+        <f>F18*F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="19">
+        <f>G18*G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>H18*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="92">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>C19*C16</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>D19*D16</f>
+        <v/>
+      </c>
+      <c r="E22" s="19">
+        <f>E19*E16</f>
+        <v/>
+      </c>
+      <c r="F22" s="19">
+        <f>F19*F16</f>
+        <v/>
+      </c>
+      <c r="G22" s="19">
+        <f>G19*G16</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>H19*H16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="92">
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="26" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1" s="92">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="14">
+        <f>(E21/C21)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="14">
+        <f>(F21/C21)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G24" s="14">
+        <f>(G21/C21)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>(H21/C21)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="92">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="n"/>
+      <c r="D25" s="30" t="n"/>
+      <c r="E25" s="31">
+        <f>(E22/C22)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>(F22/C22)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>(G22/C22)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>(H22/C22)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="92"/>
+    <row r="27" ht="16.5" customHeight="1" s="92"/>
+    <row r="28" ht="16.5" customHeight="1" s="92">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="C28" s="93" t="n"/>
+      <c r="D28" s="93" t="n"/>
+      <c r="E28" s="93" t="n"/>
+      <c r="F28" s="93" t="n"/>
+      <c r="G28" s="93" t="n"/>
+      <c r="H28" s="35" t="n">
+        <v>95</v>
+      </c>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1" s="92">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D29" s="45" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E29" s="45" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F29" s="45" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G29" s="45" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H29" s="46" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="30" ht="16.5" customHeight="1" s="92">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D30" s="40">
+        <f>(C30*C31) + C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="40">
+        <f>(D30*D31) + D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="40">
+        <f>(E30*E31) + E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="40">
+        <f>(F30*F31) + F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="41">
+        <f>(G30*G31) + G30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="92">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="44" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C31" s="58" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="E31" s="58" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="F31" s="58" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G31" s="58" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H31" s="43" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="92">
+      <c r="B32" s="44" t="n"/>
+      <c r="C32" s="45" t="n"/>
+      <c r="D32" s="45" t="n"/>
+      <c r="E32" s="45" t="n"/>
+      <c r="F32" s="45" t="n"/>
+      <c r="G32" s="45" t="n"/>
+      <c r="H32" s="46" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1" s="92">
+      <c r="B33" s="44" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="n">
+        <v>532</v>
+      </c>
+      <c r="D33" s="47">
+        <f>D30*D38</f>
+        <v/>
+      </c>
+      <c r="E33" s="47">
+        <f>E30*E38</f>
+        <v/>
+      </c>
+      <c r="F33" s="47">
+        <f>F30*F38</f>
+        <v/>
+      </c>
+      <c r="G33" s="47">
+        <f>G30*G38</f>
+        <v/>
+      </c>
+      <c r="H33" s="48">
+        <f>H30*H38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="16.5" customHeight="1" s="92">
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D34" s="49">
+        <f>(D33-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="E34" s="49">
+        <f>(E33-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="F34" s="49">
+        <f>(F33-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="G34" s="49">
+        <f>(G33-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="H34" s="50">
+        <f>(H33-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="16.5" customHeight="1" s="92">
+      <c r="B35" s="44" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="49" t="n"/>
+      <c r="E35" s="49" t="n"/>
+      <c r="F35" s="49" t="n"/>
+      <c r="G35" s="49" t="n"/>
+      <c r="H35" s="50" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1" s="92">
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C36" s="40" t="n">
+        <v>532</v>
+      </c>
+      <c r="D36" s="40" t="n">
+        <v>656</v>
+      </c>
+      <c r="E36" s="40" t="n">
+        <v>789</v>
+      </c>
+      <c r="F36" s="40" t="n">
+        <v>931</v>
+      </c>
+      <c r="G36" s="49" t="n"/>
+      <c r="H36" s="50" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1" s="92">
+      <c r="B37" s="44" t="n"/>
+      <c r="C37" s="45" t="n"/>
+      <c r="D37" s="45" t="n"/>
+      <c r="E37" s="45" t="n"/>
+      <c r="F37" s="45" t="n"/>
+      <c r="G37" s="45" t="n"/>
+      <c r="H37" s="46" t="n"/>
+    </row>
+    <row r="38" ht="16.5" customHeight="1" s="92">
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C38" s="49">
+        <f>C33/C30</f>
+        <v/>
+      </c>
+      <c r="D38" s="58" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="E38" s="58" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F38" s="58" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="G38" s="58" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="H38" s="43" t="n">
+        <v>0.235</v>
+      </c>
+    </row>
+    <row r="39" ht="16.5" customHeight="1" s="92">
+      <c r="B39" s="44" t="n"/>
+      <c r="C39" s="45" t="n"/>
+      <c r="D39" s="45" t="n"/>
+      <c r="E39" s="45" t="n"/>
+      <c r="F39" s="45" t="n"/>
+      <c r="G39" s="45" t="n"/>
+      <c r="H39" s="46" t="n"/>
+    </row>
+    <row r="40" ht="16.5" customHeight="1" s="92">
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C33/H28</f>
+        <v/>
+      </c>
+      <c r="D40" s="51">
+        <f>D33/H28</f>
+        <v/>
+      </c>
+      <c r="E40" s="51">
+        <f>E33/H28</f>
+        <v/>
+      </c>
+      <c r="F40" s="51">
+        <f>F33/H28</f>
+        <v/>
+      </c>
+      <c r="G40" s="51">
+        <f>G33/H28</f>
+        <v/>
+      </c>
+      <c r="H40" s="52">
+        <f>H33/H28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1" s="92">
+      <c r="B41" s="44" t="n"/>
+      <c r="C41" s="45" t="n"/>
+      <c r="D41" s="45" t="n"/>
+      <c r="E41" s="45" t="n"/>
+      <c r="F41" s="45" t="n"/>
+      <c r="G41" s="45" t="n"/>
+      <c r="H41" s="46" t="n"/>
+    </row>
+    <row r="42" ht="16.5" customHeight="1" s="92">
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n">
+        <v>11</v>
+      </c>
+      <c r="D42" s="55" t="n">
+        <v>11</v>
+      </c>
+      <c r="E42" s="55" t="n">
+        <v>11</v>
+      </c>
+      <c r="F42" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="G42" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="H42" s="56" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" ht="16.5" customHeight="1" s="92">
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C43" s="55" t="n">
+        <v>15</v>
+      </c>
+      <c r="D43" s="55" t="n">
+        <v>14</v>
+      </c>
+      <c r="E43" s="55" t="n">
+        <v>14</v>
+      </c>
+      <c r="F43" s="55" t="n">
+        <v>13</v>
+      </c>
+      <c r="G43" s="55" t="n">
+        <v>13</v>
+      </c>
+      <c r="H43" s="56" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" ht="16.5" customHeight="1" s="92">
+      <c r="B44" s="44" t="n"/>
+      <c r="C44" s="55" t="n"/>
+      <c r="D44" s="55" t="n"/>
+      <c r="E44" s="55" t="n"/>
+      <c r="F44" s="55" t="n"/>
+      <c r="G44" s="55" t="n"/>
+      <c r="H44" s="56" t="n"/>
+    </row>
+    <row r="45" ht="16.5" customHeight="1" s="92">
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C45" s="47">
+        <f>C42*C40</f>
+        <v/>
+      </c>
+      <c r="D45" s="47">
+        <f>D42*D40</f>
+        <v/>
+      </c>
+      <c r="E45" s="47">
+        <f>E42*E40</f>
+        <v/>
+      </c>
+      <c r="F45" s="47">
+        <f>F42*F40</f>
+        <v/>
+      </c>
+      <c r="G45" s="47">
+        <f>G42*G40</f>
+        <v/>
+      </c>
+      <c r="H45" s="57">
+        <f>H42*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1" s="92">
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C46" s="47">
+        <f>C43*C40</f>
+        <v/>
+      </c>
+      <c r="D46" s="47">
+        <f>D43*D40</f>
+        <v/>
+      </c>
+      <c r="E46" s="47">
+        <f>E43*E40</f>
+        <v/>
+      </c>
+      <c r="F46" s="47">
+        <f>F43*F40</f>
+        <v/>
+      </c>
+      <c r="G46" s="47">
+        <f>G43*G40</f>
+        <v/>
+      </c>
+      <c r="H46" s="57">
+        <f>H43*H40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1" s="92">
+      <c r="B47" s="44" t="n"/>
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="45" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="45" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="46" t="n"/>
+    </row>
+    <row r="48" ht="16.5" customHeight="1" s="92">
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C48" s="55" t="n"/>
+      <c r="D48" s="55" t="n"/>
+      <c r="E48" s="58">
+        <f>(E45/C45)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F48" s="58">
+        <f>(F45/C45)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G48" s="58">
+        <f>(G45/C45)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H48" s="59">
+        <f>(H45/C45)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1" s="92">
+      <c r="B49" s="60" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="n"/>
+      <c r="D49" s="61" t="n"/>
+      <c r="E49" s="62">
+        <f>(E46/C46)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F49" s="62">
+        <f>(F46/C46)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G49" s="62">
+        <f>(G46/C46)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H49" s="63">
+        <f>(H46/C46)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1" s="92"/>
+    <row r="51" ht="16.5" customHeight="1" s="92"/>
+    <row r="52" ht="16.5" customHeight="1" s="92">
+      <c r="A52" s="3" t="n"/>
+      <c r="B52" s="64" t="inlineStr">
+        <is>
+          <t>Bear Case</t>
+        </is>
+      </c>
+      <c r="C52" s="93" t="n"/>
+      <c r="D52" s="93" t="n"/>
+      <c r="E52" s="93" t="n"/>
+      <c r="F52" s="93" t="n"/>
+      <c r="G52" s="93" t="n"/>
+      <c r="H52" s="65" t="n">
+        <v>95</v>
+      </c>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+    </row>
+    <row r="53" ht="16.5" customHeight="1" s="92">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="74" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="C53" s="67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D53" s="67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E53" s="67" t="n">
+        <v>2028</v>
+      </c>
+      <c r="F53" s="67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="G53" s="67" t="n">
+        <v>2030</v>
+      </c>
+      <c r="H53" s="68" t="n">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="54" ht="16.5" customHeight="1" s="92">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="74" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>2550</v>
+      </c>
+      <c r="D54" s="70">
+        <f>(C54*C55) + C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="70">
+        <f>(D54*D55) + D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="70">
+        <f>(E54*E55) + E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="70">
+        <f>(F54*F55) + F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="71">
+        <f>(G54*G55) + G54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16.5" customHeight="1" s="92">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="74" t="inlineStr">
+        <is>
+          <t>Revenue G</t>
+        </is>
+      </c>
+      <c r="C55" s="86" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D55" s="86" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E55" s="86" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F55" s="86" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G55" s="86" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H55" s="73" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="56" ht="16.5" customHeight="1" s="92">
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="83" t="n"/>
+      <c r="E56" s="83" t="n"/>
+      <c r="F56" s="83" t="n"/>
+      <c r="G56" s="83" t="n"/>
+      <c r="H56" s="84" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1" s="92">
+      <c r="B57" s="74" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="C57" s="77" t="n">
+        <v>532</v>
+      </c>
+      <c r="D57" s="77">
+        <f>D54*D62</f>
+        <v/>
+      </c>
+      <c r="E57" s="77">
+        <f>E54*E62</f>
+        <v/>
+      </c>
+      <c r="F57" s="77">
+        <f>F54*F62</f>
+        <v/>
+      </c>
+      <c r="G57" s="77">
+        <f>G54*G62</f>
+        <v/>
+      </c>
+      <c r="H57" s="78">
+        <f>H54*H62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="16.5" customHeight="1" s="92">
+      <c r="B58" s="74" t="inlineStr">
+        <is>
+          <t>Net Income G</t>
+        </is>
+      </c>
+      <c r="C58" s="86" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D58" s="79">
+        <f>(D57-C57)/C57</f>
+        <v/>
+      </c>
+      <c r="E58" s="79">
+        <f>(E57-D57)/D57</f>
+        <v/>
+      </c>
+      <c r="F58" s="79">
+        <f>(F57-E57)/E57</f>
+        <v/>
+      </c>
+      <c r="G58" s="79">
+        <f>(G57-F57)/F57</f>
+        <v/>
+      </c>
+      <c r="H58" s="80">
+        <f>(H57-G57)/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="16.5" customHeight="1" s="92">
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
+      <c r="H59" s="80" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1" s="92">
+      <c r="B60" s="74" t="inlineStr">
+        <is>
+          <t>Analyst Est</t>
+        </is>
+      </c>
+      <c r="C60" s="70" t="n">
+        <v>532</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>656</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>789</v>
+      </c>
+      <c r="F60" s="70" t="n">
+        <v>931</v>
+      </c>
+      <c r="G60" s="79" t="n"/>
+      <c r="H60" s="80" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1" s="92">
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="83" t="n"/>
+      <c r="E61" s="83" t="n"/>
+      <c r="F61" s="83" t="n"/>
+      <c r="G61" s="83" t="n"/>
+      <c r="H61" s="84" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1" s="92">
+      <c r="B62" s="74" t="inlineStr">
+        <is>
+          <t>NI Margins</t>
+        </is>
+      </c>
+      <c r="C62" s="79">
+        <f>C57/C54</f>
+        <v/>
+      </c>
+      <c r="D62" s="86" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="E62" s="86" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="F62" s="86" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G62" s="86" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="H62" s="73" t="n">
+        <v>0.215</v>
+      </c>
+    </row>
+    <row r="63" ht="16.5" customHeight="1" s="92">
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="83" t="n"/>
+      <c r="D63" s="83" t="n"/>
+      <c r="E63" s="83" t="n"/>
+      <c r="F63" s="83" t="n"/>
+      <c r="G63" s="83" t="n"/>
+      <c r="H63" s="84" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1" s="92">
+      <c r="B64" s="74" t="inlineStr">
+        <is>
+          <t>EPS</t>
+        </is>
+      </c>
+      <c r="C64" s="81">
+        <f>C57/H52</f>
+        <v/>
+      </c>
+      <c r="D64" s="81">
+        <f>D57/H52</f>
+        <v/>
+      </c>
+      <c r="E64" s="81">
+        <f>E57/H52</f>
+        <v/>
+      </c>
+      <c r="F64" s="81">
+        <f>F57/H52</f>
+        <v/>
+      </c>
+      <c r="G64" s="81">
+        <f>G57/H52</f>
+        <v/>
+      </c>
+      <c r="H64" s="82">
+        <f>H57/H52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16.5" customHeight="1" s="92">
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="83" t="n"/>
+      <c r="D65" s="83" t="n"/>
+      <c r="E65" s="83" t="n"/>
+      <c r="F65" s="83" t="n"/>
+      <c r="G65" s="83" t="n"/>
+      <c r="H65" s="84" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1" s="92">
+      <c r="B66" s="74" t="inlineStr">
+        <is>
+          <t>PE Low Est</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="D66" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="E66" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="F66" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="G66" s="83" t="n">
+        <v>7</v>
+      </c>
+      <c r="H66" s="84" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="67" ht="16.5" customHeight="1" s="92">
+      <c r="B67" s="74" t="inlineStr">
+        <is>
+          <t>PE High Est</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="D67" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="E67" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="F67" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="G67" s="83" t="n">
+        <v>9</v>
+      </c>
+      <c r="H67" s="84" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" ht="16.5" customHeight="1" s="92">
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="83" t="n"/>
+      <c r="D68" s="83" t="n"/>
+      <c r="E68" s="83" t="n"/>
+      <c r="F68" s="83" t="n"/>
+      <c r="G68" s="83" t="n"/>
+      <c r="H68" s="84" t="n"/>
+    </row>
+    <row r="69" ht="16.5" customHeight="1" s="92">
+      <c r="B69" s="74" t="inlineStr">
+        <is>
+          <t>Share Price Low</t>
+        </is>
+      </c>
+      <c r="C69" s="77">
+        <f>C66*C64</f>
+        <v/>
+      </c>
+      <c r="D69" s="77">
+        <f>D66*D64</f>
+        <v/>
+      </c>
+      <c r="E69" s="77">
+        <f>E66*E64</f>
+        <v/>
+      </c>
+      <c r="F69" s="77">
+        <f>F66*F64</f>
+        <v/>
+      </c>
+      <c r="G69" s="77">
+        <f>G66*G64</f>
+        <v/>
+      </c>
+      <c r="H69" s="85">
+        <f>H66*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="16.5" customHeight="1" s="92">
+      <c r="B70" s="74" t="inlineStr">
+        <is>
+          <t>Share Price High</t>
+        </is>
+      </c>
+      <c r="C70" s="77">
+        <f>C67*C64</f>
+        <v/>
+      </c>
+      <c r="D70" s="77">
+        <f>D67*D64</f>
+        <v/>
+      </c>
+      <c r="E70" s="77">
+        <f>E67*E64</f>
+        <v/>
+      </c>
+      <c r="F70" s="77">
+        <f>F67*F64</f>
+        <v/>
+      </c>
+      <c r="G70" s="77">
+        <f>G67*G64</f>
+        <v/>
+      </c>
+      <c r="H70" s="85">
+        <f>H67*H64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="16.5" customHeight="1" s="92">
+      <c r="B71" s="74" t="n"/>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
+      <c r="E71" s="83" t="n"/>
+      <c r="F71" s="83" t="n"/>
+      <c r="G71" s="83" t="n"/>
+      <c r="H71" s="84" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1" s="92">
+      <c r="B72" s="74" t="inlineStr">
+        <is>
+          <t>CAGR Low</t>
+        </is>
+      </c>
+      <c r="C72" s="83" t="n"/>
+      <c r="D72" s="83" t="n"/>
+      <c r="E72" s="86">
+        <f>(E69/C69)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F72" s="86">
+        <f>(F69/C69)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G72" s="86">
+        <f>(G69/C69)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H72" s="87">
+        <f>(H69/C69)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="16.5" customHeight="1" s="92">
+      <c r="B73" s="88" t="inlineStr">
+        <is>
+          <t>CAGR High</t>
+        </is>
+      </c>
+      <c r="C73" s="89" t="n"/>
+      <c r="D73" s="89" t="n"/>
+      <c r="E73" s="90">
+        <f>(E70/C70)^(1/2)-1</f>
+        <v/>
+      </c>
+      <c r="F73" s="90">
+        <f>(F70/C70)^(1/3)-1</f>
+        <v/>
+      </c>
+      <c r="G73" s="90">
+        <f>(G70/C70)^(1/4)-1</f>
+        <v/>
+      </c>
+      <c r="H73" s="91">
+        <f>(H70/C70)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16.5" customHeight="1" s="92"/>
+    <row r="75" ht="16.5" customHeight="1" s="92"/>
+    <row r="76" ht="16.5" customHeight="1" s="92"/>
+    <row r="77" ht="16.5" customHeight="1" s="92"/>
+    <row r="78" ht="16.5" customHeight="1" s="92"/>
+    <row r="79" ht="16.5" customHeight="1" s="92"/>
+    <row r="80" ht="16.5" customHeight="1" s="92"/>
+    <row r="81" ht="16.5" customHeight="1" s="92"/>
+    <row r="82" ht="16.5" customHeight="1" s="92"/>
+    <row r="83" ht="16.5" customHeight="1" s="92"/>
+    <row r="84" ht="16.5" customHeight="1" s="92"/>
+    <row r="85" ht="16.5" customHeight="1" s="92"/>
+    <row r="86" ht="16.5" customHeight="1" s="92"/>
+    <row r="87" ht="16.5" customHeight="1" s="92"/>
+    <row r="88" ht="16.5" customHeight="1" s="92"/>
+    <row r="89" ht="16.5" customHeight="1" s="92"/>
+    <row r="90" ht="16.5" customHeight="1" s="92"/>
+    <row r="91" ht="16.5" customHeight="1" s="92"/>
+    <row r="92" ht="16.5" customHeight="1" s="92"/>
+    <row r="93" ht="16.5" customHeight="1" s="92"/>
+    <row r="94" ht="16.5" customHeight="1" s="92"/>
+    <row r="95" ht="16.5" customHeight="1" s="92"/>
+    <row r="96" ht="16.5" customHeight="1" s="92"/>
+    <row r="97" ht="16.5" customHeight="1" s="92"/>
+    <row r="98" ht="16.5" customHeight="1" s="92"/>
+    <row r="99" ht="16.5" customHeight="1" s="92"/>
+    <row r="100" ht="16.5" customHeight="1" s="92"/>
+    <row r="101" ht="16.5" customHeight="1" s="92"/>
+    <row r="102" ht="16.5" customHeight="1" s="92"/>
+    <row r="103" ht="16.5" customHeight="1" s="92"/>
+    <row r="104" ht="16.5" customHeight="1" s="92"/>
+    <row r="105" ht="16.5" customHeight="1" s="92"/>
+    <row r="106" ht="16.5" customHeight="1" s="92"/>
+    <row r="107" ht="16.5" customHeight="1" s="92"/>
+    <row r="108" ht="16.5" customHeight="1" s="92"/>
+    <row r="109" ht="16.5" customHeight="1" s="92"/>
+    <row r="110" ht="16.5" customHeight="1" s="92"/>
+    <row r="111" ht="16.5" customHeight="1" s="92"/>
+    <row r="112" ht="16.5" customHeight="1" s="92"/>
+    <row r="113" ht="16.5" customHeight="1" s="92"/>
+    <row r="114" ht="16.5" customHeight="1" s="92"/>
+    <row r="115" ht="16.5" customHeight="1" s="92"/>
+    <row r="116" ht="16.5" customHeight="1" s="92"/>
+    <row r="117" ht="16.5" customHeight="1" s="92"/>
+    <row r="118" ht="16.5" customHeight="1" s="92"/>
+    <row r="119" ht="16.5" customHeight="1" s="92"/>
+    <row r="120" ht="16.5" customHeight="1" s="92"/>
+    <row r="121" ht="16.5" customHeight="1" s="92"/>
+    <row r="122" ht="16.5" customHeight="1" s="92"/>
+    <row r="123" ht="16.5" customHeight="1" s="92"/>
+    <row r="124" ht="16.5" customHeight="1" s="92"/>
+    <row r="125" ht="16.5" customHeight="1" s="92"/>
+    <row r="126" ht="16.5" customHeight="1" s="92"/>
+    <row r="127" ht="16.5" customHeight="1" s="92"/>
+    <row r="128" ht="16.5" customHeight="1" s="92"/>
+    <row r="129" ht="16.5" customHeight="1" s="92"/>
+    <row r="130" ht="16.5" customHeight="1" s="92"/>
+    <row r="131" ht="16.5" customHeight="1" s="92"/>
+    <row r="132" ht="16.5" customHeight="1" s="92"/>
+    <row r="133" ht="16.5" customHeight="1" s="92"/>
+    <row r="134" ht="16.5" customHeight="1" s="92"/>
+    <row r="135" ht="16.5" customHeight="1" s="92"/>
+    <row r="136" ht="16.5" customHeight="1" s="92"/>
+    <row r="137" ht="16.5" customHeight="1" s="92"/>
+    <row r="138" ht="16.5" customHeight="1" s="92"/>
+    <row r="139" ht="16.5" customHeight="1" s="92"/>
+    <row r="140" ht="16.5" customHeight="1" s="92"/>
+    <row r="141" ht="16.5" customHeight="1" s="92"/>
+    <row r="142" ht="16.5" customHeight="1" s="92"/>
+    <row r="143" ht="16.5" customHeight="1" s="92"/>
+    <row r="144" ht="16.5" customHeight="1" s="92"/>
+    <row r="145" ht="16.5" customHeight="1" s="92"/>
+    <row r="146" ht="16.5" customHeight="1" s="92"/>
+    <row r="147" ht="16.5" customHeight="1" s="92"/>
+    <row r="148" ht="16.5" customHeight="1" s="92"/>
+    <row r="149" ht="16.5" customHeight="1" s="92"/>
+    <row r="150" ht="16.5" customHeight="1" s="92"/>
+    <row r="151" ht="16.5" customHeight="1" s="92"/>
+    <row r="152" ht="16.5" customHeight="1" s="92"/>
+    <row r="153" ht="16.5" customHeight="1" s="92"/>
+    <row r="154" ht="16.5" customHeight="1" s="92"/>
+    <row r="155" ht="16.5" customHeight="1" s="92"/>
+    <row r="156" ht="16.5" customHeight="1" s="92"/>
+    <row r="157" ht="16.5" customHeight="1" s="92"/>
+    <row r="158" ht="16.5" customHeight="1" s="92"/>
+    <row r="159" ht="16.5" customHeight="1" s="92"/>
+    <row r="160" ht="16.5" customHeight="1" s="92"/>
+    <row r="161" ht="16.5" customHeight="1" s="92"/>
+    <row r="162" ht="16.5" customHeight="1" s="92"/>
+    <row r="163" ht="16.5" customHeight="1" s="92"/>
+    <row r="164" ht="16.5" customHeight="1" s="92"/>
+    <row r="165" ht="16.5" customHeight="1" s="92"/>
+    <row r="166" ht="16.5" customHeight="1" s="92"/>
+    <row r="167" ht="16.5" customHeight="1" s="92"/>
+    <row r="168" ht="16.5" customHeight="1" s="92"/>
+    <row r="169" ht="16.5" customHeight="1" s="92"/>
+    <row r="170" ht="16.5" customHeight="1" s="92"/>
+    <row r="171" ht="16.5" customHeight="1" s="92"/>
+    <row r="172" ht="16.5" customHeight="1" s="92"/>
+    <row r="173" ht="16.5" customHeight="1" s="92"/>
+    <row r="174" ht="16.5" customHeight="1" s="92"/>
+    <row r="175" ht="16.5" customHeight="1" s="92"/>
+    <row r="176" ht="16.5" customHeight="1" s="92"/>
+    <row r="177" ht="16.5" customHeight="1" s="92"/>
+    <row r="178" ht="16.5" customHeight="1" s="92"/>
+    <row r="179" ht="16.5" customHeight="1" s="92"/>
+    <row r="180" ht="16.5" customHeight="1" s="92"/>
+    <row r="181" ht="16.5" customHeight="1" s="92"/>
+    <row r="182" ht="16.5" customHeight="1" s="92"/>
+    <row r="183" ht="16.5" customHeight="1" s="92"/>
+    <row r="184" ht="16.5" customHeight="1" s="92"/>
+    <row r="185" ht="16.5" customHeight="1" s="92"/>
+    <row r="186" ht="16.5" customHeight="1" s="92"/>
+    <row r="187" ht="16.5" customHeight="1" s="92"/>
+    <row r="188" ht="16.5" customHeight="1" s="92"/>
+    <row r="189" ht="16.5" customHeight="1" s="92"/>
+    <row r="190" ht="16.5" customHeight="1" s="92"/>
+    <row r="191" ht="16.5" customHeight="1" s="92"/>
+    <row r="192" ht="16.5" customHeight="1" s="92"/>
+    <row r="193" ht="16.5" customHeight="1" s="92"/>
+    <row r="194" ht="16.5" customHeight="1" s="92"/>
+    <row r="195" ht="16.5" customHeight="1" s="92"/>
+    <row r="196" ht="16.5" customHeight="1" s="92"/>
+    <row r="197" ht="16.5" customHeight="1" s="92"/>
+    <row r="198" ht="16.5" customHeight="1" s="92"/>
+    <row r="199" ht="16.5" customHeight="1" s="92"/>
+    <row r="200" ht="16.5" customHeight="1" s="92"/>
+    <row r="201" ht="16.5" customHeight="1" s="92"/>
+    <row r="202" ht="16.5" customHeight="1" s="92"/>
+    <row r="203" ht="16.5" customHeight="1" s="92"/>
+    <row r="204" ht="16.5" customHeight="1" s="92"/>
+    <row r="205" ht="16.5" customHeight="1" s="92"/>
+    <row r="206" ht="16.5" customHeight="1" s="92"/>
+    <row r="207" ht="16.5" customHeight="1" s="92"/>
+    <row r="208" ht="16.5" customHeight="1" s="92"/>
+    <row r="209" ht="16.5" customHeight="1" s="92"/>
+    <row r="210" ht="16.5" customHeight="1" s="92"/>
+    <row r="211" ht="16.5" customHeight="1" s="92"/>
+    <row r="212" ht="16.5" customHeight="1" s="92"/>
+    <row r="213" ht="16.5" customHeight="1" s="92"/>
+    <row r="214" ht="16.5" customHeight="1" s="92"/>
+    <row r="215" ht="16.5" customHeight="1" s="92"/>
+    <row r="216" ht="16.5" customHeight="1" s="92"/>
+    <row r="217" ht="16.5" customHeight="1" s="92"/>
+    <row r="218" ht="16.5" customHeight="1" s="92"/>
+    <row r="219" ht="16.5" customHeight="1" s="92"/>
+    <row r="220" ht="16.5" customHeight="1" s="92"/>
+    <row r="221" ht="16.5" customHeight="1" s="92"/>
+    <row r="222" ht="16.5" customHeight="1" s="92"/>
+    <row r="223" ht="16.5" customHeight="1" s="92"/>
+    <row r="224" ht="16.5" customHeight="1" s="92"/>
+    <row r="225" ht="16.5" customHeight="1" s="92"/>
+    <row r="226" ht="16.5" customHeight="1" s="92"/>
+    <row r="227" ht="16.5" customHeight="1" s="92"/>
+    <row r="228" ht="16.5" customHeight="1" s="92"/>
+    <row r="229" ht="16.5" customHeight="1" s="92"/>
+    <row r="230" ht="16.5" customHeight="1" s="92"/>
+    <row r="231" ht="16.5" customHeight="1" s="92"/>
+    <row r="232" ht="16.5" customHeight="1" s="92"/>
+    <row r="233" ht="16.5" customHeight="1" s="92"/>
+    <row r="234" ht="16.5" customHeight="1" s="92"/>
+    <row r="235" ht="16.5" customHeight="1" s="92"/>
+    <row r="236" ht="16.5" customHeight="1" s="92"/>
+    <row r="237" ht="16.5" customHeight="1" s="92"/>
+    <row r="238" ht="16.5" customHeight="1" s="92"/>
+    <row r="239" ht="16.5" customHeight="1" s="92"/>
+    <row r="240" ht="16.5" customHeight="1" s="92"/>
+    <row r="241" ht="16.5" customHeight="1" s="92"/>
+    <row r="242" ht="16.5" customHeight="1" s="92"/>
+    <row r="243" ht="16.5" customHeight="1" s="92"/>
+    <row r="244" ht="16.5" customHeight="1" s="92"/>
+    <row r="245" ht="16.5" customHeight="1" s="92"/>
+    <row r="246" ht="16.5" customHeight="1" s="92"/>
+    <row r="247" ht="16.5" customHeight="1" s="92"/>
+    <row r="248" ht="16.5" customHeight="1" s="92"/>
+    <row r="249" ht="16.5" customHeight="1" s="92"/>
+    <row r="250" ht="16.5" customHeight="1" s="92"/>
+    <row r="251" ht="16.5" customHeight="1" s="92"/>
+    <row r="252" ht="16.5" customHeight="1" s="92"/>
+    <row r="253" ht="16.5" customHeight="1" s="92"/>
+    <row r="254" ht="16.5" customHeight="1" s="92"/>
+    <row r="255" ht="16.5" customHeight="1" s="92"/>
+    <row r="256" ht="16.5" customHeight="1" s="92"/>
+    <row r="257" ht="16.5" customHeight="1" s="92"/>
+    <row r="258" ht="16.5" customHeight="1" s="92"/>
+    <row r="259" ht="16.5" customHeight="1" s="92"/>
+    <row r="260" ht="16.5" customHeight="1" s="92"/>
+    <row r="261" ht="16.5" customHeight="1" s="92"/>
+    <row r="262" ht="16.5" customHeight="1" s="92"/>
+    <row r="263" ht="16.5" customHeight="1" s="92"/>
+    <row r="264" ht="16.5" customHeight="1" s="92"/>
+    <row r="265" ht="16.5" customHeight="1" s="92"/>
+    <row r="266" ht="16.5" customHeight="1" s="92"/>
+    <row r="267" ht="16.5" customHeight="1" s="92"/>
+    <row r="268" ht="16.5" customHeight="1" s="92"/>
+    <row r="269" ht="16.5" customHeight="1" s="92"/>
+    <row r="270" ht="16.5" customHeight="1" s="92"/>
+    <row r="271" ht="16.5" customHeight="1" s="92"/>
+    <row r="272" ht="16.5" customHeight="1" s="92"/>
+    <row r="273" ht="16.5" customHeight="1" s="92"/>
+    <row r="274" ht="16.5" customHeight="1" s="92"/>
+    <row r="275" ht="16.5" customHeight="1" s="92"/>
+    <row r="276" ht="16.5" customHeight="1" s="92"/>
+    <row r="277" ht="16.5" customHeight="1" s="92"/>
+    <row r="278" ht="16.5" customHeight="1" s="92"/>
+    <row r="279" ht="16.5" customHeight="1" s="92"/>
+    <row r="280" ht="16.5" customHeight="1" s="92"/>
+    <row r="281" ht="16.5" customHeight="1" s="92"/>
+    <row r="282" ht="16.5" customHeight="1" s="92"/>
+    <row r="283" ht="16.5" customHeight="1" s="92"/>
+    <row r="284" ht="16.5" customHeight="1" s="92"/>
+    <row r="285" ht="16.5" customHeight="1" s="92"/>
+    <row r="286" ht="16.5" customHeight="1" s="92"/>
+    <row r="287" ht="16.5" customHeight="1" s="92"/>
+    <row r="288" ht="16.5" customHeight="1" s="92"/>
+    <row r="289" ht="16.5" customHeight="1" s="92"/>
+    <row r="290" ht="16.5" customHeight="1" s="92"/>
+    <row r="291" ht="16.5" customHeight="1" s="92"/>
+    <row r="292" ht="16.5" customHeight="1" s="92"/>
+    <row r="293" ht="16.5" customHeight="1" s="92"/>
+    <row r="294" ht="16.5" customHeight="1" s="92"/>
+    <row r="295" ht="16.5" customHeight="1" s="92"/>
+    <row r="296" ht="16.5" customHeight="1" s="92"/>
+    <row r="297" ht="16.5" customHeight="1" s="92"/>
+    <row r="298" ht="16.5" customHeight="1" s="92"/>
+    <row r="299" ht="16.5" customHeight="1" s="92"/>
+    <row r="300" ht="16.5" customHeight="1" s="92"/>
+    <row r="301" ht="16.5" customHeight="1" s="92"/>
+    <row r="302" ht="16.5" customHeight="1" s="92"/>
+    <row r="303" ht="16.5" customHeight="1" s="92"/>
+    <row r="304" ht="16.5" customHeight="1" s="92"/>
+    <row r="305" ht="16.5" customHeight="1" s="92"/>
+    <row r="306" ht="16.5" customHeight="1" s="92"/>
+    <row r="307" ht="16.5" customHeight="1" s="92"/>
+    <row r="308" ht="16.5" customHeight="1" s="92"/>
+    <row r="309" ht="16.5" customHeight="1" s="92"/>
+    <row r="310" ht="16.5" customHeight="1" s="92"/>
+    <row r="311" ht="16.5" customHeight="1" s="92"/>
+    <row r="312" ht="16.5" customHeight="1" s="92"/>
+    <row r="313" ht="16.5" customHeight="1" s="92"/>
+    <row r="314" ht="16.5" customHeight="1" s="92"/>
+    <row r="315" ht="16.5" customHeight="1" s="92"/>
+    <row r="316" ht="16.5" customHeight="1" s="92"/>
+    <row r="317" ht="16.5" customHeight="1" s="92"/>
+    <row r="318" ht="16.5" customHeight="1" s="92"/>
+    <row r="319" ht="16.5" customHeight="1" s="92"/>
+    <row r="320" ht="16.5" customHeight="1" s="92"/>
+    <row r="321" ht="16.5" customHeight="1" s="92"/>
+    <row r="322" ht="16.5" customHeight="1" s="92"/>
+    <row r="323" ht="16.5" customHeight="1" s="92"/>
+    <row r="324" ht="16.5" customHeight="1" s="92"/>
+    <row r="325" ht="16.5" customHeight="1" s="92"/>
+    <row r="326" ht="16.5" customHeight="1" s="92"/>
+    <row r="327" ht="16.5" customHeight="1" s="92"/>
+    <row r="328" ht="16.5" customHeight="1" s="92"/>
+    <row r="329" ht="16.5" customHeight="1" s="92"/>
+    <row r="330" ht="16.5" customHeight="1" s="92"/>
+    <row r="331" ht="16.5" customHeight="1" s="92"/>
+    <row r="332" ht="16.5" customHeight="1" s="92"/>
+    <row r="333" ht="16.5" customHeight="1" s="92"/>
+    <row r="334" ht="16.5" customHeight="1" s="92"/>
+    <row r="335" ht="16.5" customHeight="1" s="92"/>
+    <row r="336" ht="16.5" customHeight="1" s="92"/>
+    <row r="337" ht="16.5" customHeight="1" s="92"/>
+    <row r="338" ht="16.5" customHeight="1" s="92"/>
+    <row r="339" ht="16.5" customHeight="1" s="92"/>
+    <row r="340" ht="16.5" customHeight="1" s="92"/>
+    <row r="341" ht="16.5" customHeight="1" s="92"/>
+    <row r="342" ht="16.5" customHeight="1" s="92"/>
+    <row r="343" ht="16.5" customHeight="1" s="92"/>
+    <row r="344" ht="16.5" customHeight="1" s="92"/>
+    <row r="345" ht="16.5" customHeight="1" s="92"/>
+    <row r="346" ht="16.5" customHeight="1" s="92"/>
+    <row r="347" ht="16.5" customHeight="1" s="92"/>
+    <row r="348" ht="16.5" customHeight="1" s="92"/>
+    <row r="349" ht="16.5" customHeight="1" s="92"/>
+    <row r="350" ht="16.5" customHeight="1" s="92"/>
+    <row r="351" ht="16.5" customHeight="1" s="92"/>
+    <row r="352" ht="16.5" customHeight="1" s="92"/>
+    <row r="353" ht="16.5" customHeight="1" s="92"/>
+    <row r="354" ht="16.5" customHeight="1" s="92"/>
+    <row r="355" ht="16.5" customHeight="1" s="92"/>
+    <row r="356" ht="16.5" customHeight="1" s="92"/>
+    <row r="357" ht="16.5" customHeight="1" s="92"/>
+    <row r="358" ht="16.5" customHeight="1" s="92"/>
+    <row r="359" ht="16.5" customHeight="1" s="92"/>
+    <row r="360" ht="16.5" customHeight="1" s="92"/>
+    <row r="361" ht="16.5" customHeight="1" s="92"/>
+    <row r="362" ht="16.5" customHeight="1" s="92"/>
+    <row r="363" ht="16.5" customHeight="1" s="92"/>
+    <row r="364" ht="16.5" customHeight="1" s="92"/>
+    <row r="365" ht="16.5" customHeight="1" s="92"/>
+    <row r="366" ht="16.5" customHeight="1" s="92"/>
+    <row r="367" ht="16.5" customHeight="1" s="92"/>
+    <row r="368" ht="16.5" customHeight="1" s="92"/>
+    <row r="369" ht="16.5" customHeight="1" s="92"/>
+    <row r="370" ht="16.5" customHeight="1" s="92"/>
+    <row r="371" ht="16.5" customHeight="1" s="92"/>
+    <row r="372" ht="16.5" customHeight="1" s="92"/>
+    <row r="373" ht="16.5" customHeight="1" s="92"/>
+    <row r="374" ht="16.5" customHeight="1" s="92"/>
+    <row r="375" ht="16.5" customHeight="1" s="92"/>
+    <row r="376" ht="16.5" customHeight="1" s="92"/>
+    <row r="377" ht="16.5" customHeight="1" s="92"/>
+    <row r="378" ht="16.5" customHeight="1" s="92"/>
+    <row r="379" ht="16.5" customHeight="1" s="92"/>
+    <row r="380" ht="16.5" customHeight="1" s="92"/>
+    <row r="381" ht="16.5" customHeight="1" s="92"/>
+    <row r="382" ht="16.5" customHeight="1" s="92"/>
+    <row r="383" ht="16.5" customHeight="1" s="92"/>
+    <row r="384" ht="16.5" customHeight="1" s="92"/>
+    <row r="385" ht="16.5" customHeight="1" s="92"/>
+    <row r="386" ht="16.5" customHeight="1" s="92"/>
+    <row r="387" ht="16.5" customHeight="1" s="92"/>
+    <row r="388" ht="16.5" customHeight="1" s="92"/>
+    <row r="389" ht="16.5" customHeight="1" s="92"/>
+    <row r="390" ht="16.5" customHeight="1" s="92"/>
+    <row r="391" ht="16.5" customHeight="1" s="92"/>
+    <row r="392" ht="16.5" customHeight="1" s="92"/>
+    <row r="393" ht="16.5" customHeight="1" s="92"/>
+    <row r="394" ht="16.5" customHeight="1" s="92"/>
+    <row r="395" ht="16.5" customHeight="1" s="92"/>
+    <row r="396" ht="16.5" customHeight="1" s="92"/>
+    <row r="397" ht="16.5" customHeight="1" s="92"/>
+    <row r="398" ht="16.5" customHeight="1" s="92"/>
+    <row r="399" ht="16.5" customHeight="1" s="92"/>
+    <row r="400" ht="16.5" customHeight="1" s="92"/>
+    <row r="401" ht="16.5" customHeight="1" s="92"/>
+    <row r="402" ht="16.5" customHeight="1" s="92"/>
+    <row r="403" ht="16.5" customHeight="1" s="92"/>
+    <row r="404" ht="16.5" customHeight="1" s="92"/>
+    <row r="405" ht="16.5" customHeight="1" s="92"/>
+    <row r="406" ht="16.5" customHeight="1" s="92"/>
+    <row r="407" ht="16.5" customHeight="1" s="92"/>
+    <row r="408" ht="16.5" customHeight="1" s="92"/>
+    <row r="409" ht="16.5" customHeight="1" s="92"/>
+    <row r="410" ht="16.5" customHeight="1" s="92"/>
+    <row r="411" ht="16.5" customHeight="1" s="92"/>
+    <row r="412" ht="16.5" customHeight="1" s="92"/>
+    <row r="413" ht="16.5" customHeight="1" s="92"/>
+    <row r="414" ht="16.5" customHeight="1" s="92"/>
+    <row r="415" ht="16.5" customHeight="1" s="92"/>
+    <row r="416" ht="16.5" customHeight="1" s="92"/>
+    <row r="417" ht="16.5" customHeight="1" s="92"/>
+    <row r="418" ht="16.5" customHeight="1" s="92"/>
+    <row r="419" ht="16.5" customHeight="1" s="92"/>
+    <row r="420" ht="16.5" customHeight="1" s="92"/>
+    <row r="421" ht="16.5" customHeight="1" s="92"/>
+    <row r="422" ht="16.5" customHeight="1" s="92"/>
+    <row r="423" ht="16.5" customHeight="1" s="92"/>
+    <row r="424" ht="16.5" customHeight="1" s="92"/>
+    <row r="425" ht="16.5" customHeight="1" s="92"/>
+    <row r="426" ht="16.5" customHeight="1" s="92"/>
+    <row r="427" ht="16.5" customHeight="1" s="92"/>
+    <row r="428" ht="16.5" customHeight="1" s="92"/>
+    <row r="429" ht="16.5" customHeight="1" s="92"/>
+    <row r="430" ht="16.5" customHeight="1" s="92"/>
+    <row r="431" ht="16.5" customHeight="1" s="92"/>
+    <row r="432" ht="16.5" customHeight="1" s="92"/>
+    <row r="433" ht="16.5" customHeight="1" s="92"/>
+    <row r="434" ht="16.5" customHeight="1" s="92"/>
+    <row r="435" ht="16.5" customHeight="1" s="92"/>
+    <row r="436" ht="16.5" customHeight="1" s="92"/>
+    <row r="437" ht="16.5" customHeight="1" s="92"/>
+    <row r="438" ht="16.5" customHeight="1" s="92"/>
+    <row r="439" ht="16.5" customHeight="1" s="92"/>
+    <row r="440" ht="16.5" customHeight="1" s="92"/>
+    <row r="441" ht="16.5" customHeight="1" s="92"/>
+    <row r="442" ht="16.5" customHeight="1" s="92"/>
+    <row r="443" ht="16.5" customHeight="1" s="92"/>
+    <row r="444" ht="16.5" customHeight="1" s="92"/>
+    <row r="445" ht="16.5" customHeight="1" s="92"/>
+    <row r="446" ht="16.5" customHeight="1" s="92"/>
+    <row r="447" ht="16.5" customHeight="1" s="92"/>
+    <row r="448" ht="16.5" customHeight="1" s="92"/>
+    <row r="449" ht="16.5" customHeight="1" s="92"/>
+    <row r="450" ht="16.5" customHeight="1" s="92"/>
+    <row r="451" ht="16.5" customHeight="1" s="92"/>
+    <row r="452" ht="16.5" customHeight="1" s="92"/>
+    <row r="453" ht="16.5" customHeight="1" s="92"/>
+    <row r="454" ht="16.5" customHeight="1" s="92"/>
+    <row r="455" ht="16.5" customHeight="1" s="92"/>
+    <row r="456" ht="16.5" customHeight="1" s="92"/>
+    <row r="457" ht="16.5" customHeight="1" s="92"/>
+    <row r="458" ht="16.5" customHeight="1" s="92"/>
+    <row r="459" ht="16.5" customHeight="1" s="92"/>
+    <row r="460" ht="16.5" customHeight="1" s="92"/>
+    <row r="461" ht="16.5" customHeight="1" s="92"/>
+    <row r="462" ht="16.5" customHeight="1" s="92"/>
+    <row r="463" ht="16.5" customHeight="1" s="92"/>
+    <row r="464" ht="16.5" customHeight="1" s="92"/>
+    <row r="465" ht="16.5" customHeight="1" s="92"/>
+    <row r="466" ht="16.5" customHeight="1" s="92"/>
+    <row r="467" ht="16.5" customHeight="1" s="92"/>
+    <row r="468" ht="16.5" customHeight="1" s="92"/>
+    <row r="469" ht="16.5" customHeight="1" s="92"/>
+    <row r="470" ht="16.5" customHeight="1" s="92"/>
+    <row r="471" ht="16.5" customHeight="1" s="92"/>
+    <row r="472" ht="16.5" customHeight="1" s="92"/>
+    <row r="473" ht="16.5" customHeight="1" s="92"/>
+    <row r="474" ht="16.5" customHeight="1" s="92"/>
+    <row r="475" ht="16.5" customHeight="1" s="92"/>
+    <row r="476" ht="16.5" customHeight="1" s="92"/>
+    <row r="477" ht="16.5" customHeight="1" s="92"/>
+    <row r="478" ht="16.5" customHeight="1" s="92"/>
+    <row r="479" ht="16.5" customHeight="1" s="92"/>
+    <row r="480" ht="16.5" customHeight="1" s="92"/>
+    <row r="481" ht="16.5" customHeight="1" s="92"/>
+    <row r="482" ht="16.5" customHeight="1" s="92"/>
+    <row r="483" ht="16.5" customHeight="1" s="92"/>
+    <row r="484" ht="16.5" customHeight="1" s="92"/>
+    <row r="485" ht="16.5" customHeight="1" s="92"/>
+    <row r="486" ht="16.5" customHeight="1" s="92"/>
+    <row r="487" ht="16.5" customHeight="1" s="92"/>
+    <row r="488" ht="16.5" customHeight="1" s="92"/>
+    <row r="489" ht="16.5" customHeight="1" s="92"/>
+    <row r="490" ht="16.5" customHeight="1" s="92"/>
+    <row r="491" ht="16.5" customHeight="1" s="92"/>
+    <row r="492" ht="16.5" customHeight="1" s="92"/>
+    <row r="493" ht="16.5" customHeight="1" s="92"/>
+    <row r="494" ht="16.5" customHeight="1" s="92"/>
+    <row r="495" ht="16.5" customHeight="1" s="92"/>
+    <row r="496" ht="16.5" customHeight="1" s="92"/>
+    <row r="497" ht="16.5" customHeight="1" s="92"/>
+    <row r="498" ht="16.5" customHeight="1" s="92"/>
+    <row r="499" ht="16.5" customHeight="1" s="92"/>
+    <row r="500" ht="16.5" customHeight="1" s="92"/>
+    <row r="501" ht="16.5" customHeight="1" s="92"/>
+    <row r="502" ht="16.5" customHeight="1" s="92"/>
+    <row r="503" ht="16.5" customHeight="1" s="92"/>
+    <row r="504" ht="16.5" customHeight="1" s="92"/>
+    <row r="505" ht="16.5" customHeight="1" s="92"/>
+    <row r="506" ht="16.5" customHeight="1" s="92"/>
+    <row r="507" ht="16.5" customHeight="1" s="92"/>
+    <row r="508" ht="16.5" customHeight="1" s="92"/>
+    <row r="509" ht="16.5" customHeight="1" s="92"/>
+    <row r="510" ht="16.5" customHeight="1" s="92"/>
+    <row r="511" ht="16.5" customHeight="1" s="92"/>
+    <row r="512" ht="16.5" customHeight="1" s="92"/>
+    <row r="513" ht="16.5" customHeight="1" s="92"/>
+    <row r="514" ht="16.5" customHeight="1" s="92"/>
+    <row r="515" ht="16.5" customHeight="1" s="92"/>
+    <row r="516" ht="16.5" customHeight="1" s="92"/>
+    <row r="517" ht="16.5" customHeight="1" s="92"/>
+    <row r="518" ht="16.5" customHeight="1" s="92"/>
+    <row r="519" ht="16.5" customHeight="1" s="92"/>
+    <row r="520" ht="16.5" customHeight="1" s="92"/>
+    <row r="521" ht="16.5" customHeight="1" s="92"/>
+    <row r="522" ht="16.5" customHeight="1" s="92"/>
+    <row r="523" ht="16.5" customHeight="1" s="92"/>
+    <row r="524" ht="16.5" customHeight="1" s="92"/>
+    <row r="525" ht="16.5" customHeight="1" s="92"/>
+    <row r="526" ht="16.5" customHeight="1" s="92"/>
+    <row r="527" ht="16.5" customHeight="1" s="92"/>
+    <row r="528" ht="16.5" customHeight="1" s="92"/>
+    <row r="529" ht="16.5" customHeight="1" s="92"/>
+    <row r="530" ht="16.5" customHeight="1" s="92"/>
+    <row r="531" ht="16.5" customHeight="1" s="92"/>
+    <row r="532" ht="16.5" customHeight="1" s="92"/>
+    <row r="533" ht="16.5" customHeight="1" s="92"/>
+    <row r="534" ht="16.5" customHeight="1" s="92"/>
+    <row r="535" ht="16.5" customHeight="1" s="92"/>
+    <row r="536" ht="16.5" customHeight="1" s="92"/>
+    <row r="537" ht="16.5" customHeight="1" s="92"/>
+    <row r="538" ht="16.5" customHeight="1" s="92"/>
+    <row r="539" ht="16.5" customHeight="1" s="92"/>
+    <row r="540" ht="16.5" customHeight="1" s="92"/>
+    <row r="541" ht="16.5" customHeight="1" s="92"/>
+    <row r="542" ht="16.5" customHeight="1" s="92"/>
+    <row r="543" ht="16.5" customHeight="1" s="92"/>
+    <row r="544" ht="16.5" customHeight="1" s="92"/>
+    <row r="545" ht="16.5" customHeight="1" s="92"/>
+    <row r="546" ht="16.5" customHeight="1" s="92"/>
+    <row r="547" ht="16.5" customHeight="1" s="92"/>
+    <row r="548" ht="16.5" customHeight="1" s="92"/>
+    <row r="549" ht="16.5" customHeight="1" s="92"/>
+    <row r="550" ht="16.5" customHeight="1" s="92"/>
+    <row r="551" ht="16.5" customHeight="1" s="92"/>
+    <row r="552" ht="16.5" customHeight="1" s="92"/>
+    <row r="553" ht="16.5" customHeight="1" s="92"/>
+    <row r="554" ht="16.5" customHeight="1" s="92"/>
+    <row r="555" ht="16.5" customHeight="1" s="92"/>
+    <row r="556" ht="16.5" customHeight="1" s="92"/>
+    <row r="557" ht="16.5" customHeight="1" s="92"/>
+    <row r="558" ht="16.5" customHeight="1" s="92"/>
+    <row r="559" ht="16.5" customHeight="1" s="92"/>
+    <row r="560" ht="16.5" customHeight="1" s="92"/>
+    <row r="561" ht="16.5" customHeight="1" s="92"/>
+    <row r="562" ht="16.5" customHeight="1" s="92"/>
+    <row r="563" ht="16.5" customHeight="1" s="92"/>
+    <row r="564" ht="16.5" customHeight="1" s="92"/>
+    <row r="565" ht="16.5" customHeight="1" s="92"/>
+    <row r="566" ht="16.5" customHeight="1" s="92"/>
+    <row r="567" ht="16.5" customHeight="1" s="92"/>
+    <row r="568" ht="16.5" customHeight="1" s="92"/>
+    <row r="569" ht="16.5" customHeight="1" s="92"/>
+    <row r="570" ht="16.5" customHeight="1" s="92"/>
+    <row r="571" ht="16.5" customHeight="1" s="92"/>
+    <row r="572" ht="16.5" customHeight="1" s="92"/>
+    <row r="573" ht="16.5" customHeight="1" s="92"/>
+    <row r="574" ht="16.5" customHeight="1" s="92"/>
+    <row r="575" ht="16.5" customHeight="1" s="92"/>
+    <row r="576" ht="16.5" customHeight="1" s="92"/>
+    <row r="577" ht="16.5" customHeight="1" s="92"/>
+    <row r="578" ht="16.5" customHeight="1" s="92"/>
+    <row r="579" ht="16.5" customHeight="1" s="92"/>
+    <row r="580" ht="16.5" customHeight="1" s="92"/>
+    <row r="581" ht="16.5" customHeight="1" s="92"/>
+    <row r="582" ht="16.5" customHeight="1" s="92"/>
+    <row r="583" ht="16.5" customHeight="1" s="92"/>
+    <row r="584" ht="16.5" customHeight="1" s="92"/>
+    <row r="585" ht="16.5" customHeight="1" s="92"/>
+    <row r="586" ht="16.5" customHeight="1" s="92"/>
+    <row r="587" ht="16.5" customHeight="1" s="92"/>
+    <row r="588" ht="16.5" customHeight="1" s="92"/>
+    <row r="589" ht="16.5" customHeight="1" s="92"/>
+    <row r="590" ht="16.5" customHeight="1" s="92"/>
+    <row r="591" ht="16.5" customHeight="1" s="92"/>
+    <row r="592" ht="16.5" customHeight="1" s="92"/>
+    <row r="593" ht="16.5" customHeight="1" s="92"/>
+    <row r="594" ht="16.5" customHeight="1" s="92"/>
+    <row r="595" ht="16.5" customHeight="1" s="92"/>
+    <row r="596" ht="16.5" customHeight="1" s="92"/>
+    <row r="597" ht="16.5" customHeight="1" s="92"/>
+    <row r="598" ht="16.5" customHeight="1" s="92"/>
+    <row r="599" ht="16.5" customHeight="1" s="92"/>
+    <row r="600" ht="16.5" customHeight="1" s="92"/>
+    <row r="601" ht="16.5" customHeight="1" s="92"/>
+    <row r="602" ht="16.5" customHeight="1" s="92"/>
+    <row r="603" ht="16.5" customHeight="1" s="92"/>
+    <row r="604" ht="16.5" customHeight="1" s="92"/>
+    <row r="605" ht="16.5" customHeight="1" s="92"/>
+    <row r="606" ht="16.5" customHeight="1" s="92"/>
+    <row r="607" ht="16.5" customHeight="1" s="92"/>
+    <row r="608" ht="16.5" customHeight="1" s="92"/>
+    <row r="609" ht="16.5" customHeight="1" s="92"/>
+    <row r="610" ht="16.5" customHeight="1" s="92"/>
+    <row r="611" ht="16.5" customHeight="1" s="92"/>
+    <row r="612" ht="16.5" customHeight="1" s="92"/>
+    <row r="613" ht="16.5" customHeight="1" s="92"/>
+    <row r="614" ht="16.5" customHeight="1" s="92"/>
+    <row r="615" ht="16.5" customHeight="1" s="92"/>
+    <row r="616" ht="16.5" customHeight="1" s="92"/>
+    <row r="617" ht="16.5" customHeight="1" s="92"/>
+    <row r="618" ht="16.5" customHeight="1" s="92"/>
+    <row r="619" ht="16.5" customHeight="1" s="92"/>
+    <row r="620" ht="16.5" customHeight="1" s="92"/>
+    <row r="621" ht="16.5" customHeight="1" s="92"/>
+    <row r="622" ht="16.5" customHeight="1" s="92"/>
+    <row r="623" ht="16.5" customHeight="1" s="92"/>
+    <row r="624" ht="16.5" customHeight="1" s="92"/>
+    <row r="625" ht="16.5" customHeight="1" s="92"/>
+    <row r="626" ht="16.5" customHeight="1" s="92"/>
+    <row r="627" ht="16.5" customHeight="1" s="92"/>
+    <row r="628" ht="16.5" customHeight="1" s="92"/>
+    <row r="629" ht="16.5" customHeight="1" s="92"/>
+    <row r="630" ht="16.5" customHeight="1" s="92"/>
+    <row r="631" ht="16.5" customHeight="1" s="92"/>
+    <row r="632" ht="16.5" customHeight="1" s="92"/>
+    <row r="633" ht="16.5" customHeight="1" s="92"/>
+    <row r="634" ht="16.5" customHeight="1" s="92"/>
+    <row r="635" ht="16.5" customHeight="1" s="92"/>
+    <row r="636" ht="16.5" customHeight="1" s="92"/>
+    <row r="637" ht="16.5" customHeight="1" s="92"/>
+    <row r="638" ht="16.5" customHeight="1" s="92"/>
+    <row r="639" ht="16.5" customHeight="1" s="92"/>
+    <row r="640" ht="16.5" customHeight="1" s="92"/>
+    <row r="641" ht="16.5" customHeight="1" s="92"/>
+    <row r="642" ht="16.5" customHeight="1" s="92"/>
+    <row r="643" ht="16.5" customHeight="1" s="92"/>
+    <row r="644" ht="16.5" customHeight="1" s="92"/>
+    <row r="645" ht="16.5" customHeight="1" s="92"/>
+    <row r="646" ht="16.5" customHeight="1" s="92"/>
+    <row r="647" ht="16.5" customHeight="1" s="92"/>
+    <row r="648" ht="16.5" customHeight="1" s="92"/>
+    <row r="649" ht="16.5" customHeight="1" s="92"/>
+    <row r="650" ht="16.5" customHeight="1" s="92"/>
+    <row r="651" ht="16.5" customHeight="1" s="92"/>
+    <row r="652" ht="16.5" customHeight="1" s="92"/>
+    <row r="653" ht="16.5" customHeight="1" s="92"/>
+    <row r="654" ht="16.5" customHeight="1" s="92"/>
+    <row r="655" ht="16.5" customHeight="1" s="92"/>
+    <row r="656" ht="16.5" customHeight="1" s="92"/>
+    <row r="657" ht="16.5" customHeight="1" s="92"/>
+    <row r="658" ht="16.5" customHeight="1" s="92"/>
+    <row r="659" ht="16.5" customHeight="1" s="92"/>
+    <row r="660" ht="16.5" customHeight="1" s="92"/>
+    <row r="661" ht="16.5" customHeight="1" s="92"/>
+    <row r="662" ht="16.5" customHeight="1" s="92"/>
+    <row r="663" ht="16.5" customHeight="1" s="92"/>
+    <row r="664" ht="16.5" customHeight="1" s="92"/>
+    <row r="665" ht="16.5" customHeight="1" s="92"/>
+    <row r="666" ht="16.5" customHeight="1" s="92"/>
+    <row r="667" ht="16.5" customHeight="1" s="92"/>
+    <row r="668" ht="16.5" customHeight="1" s="92"/>
+    <row r="669" ht="16.5" customHeight="1" s="92"/>
+    <row r="670" ht="16.5" customHeight="1" s="92"/>
+    <row r="671" ht="16.5" customHeight="1" s="92"/>
+    <row r="672" ht="16.5" customHeight="1" s="92"/>
+    <row r="673" ht="16.5" customHeight="1" s="92"/>
+    <row r="674" ht="16.5" customHeight="1" s="92"/>
+    <row r="675" ht="16.5" customHeight="1" s="92"/>
+    <row r="676" ht="16.5" customHeight="1" s="92"/>
+    <row r="677" ht="16.5" customHeight="1" s="92"/>
+    <row r="678" ht="16.5" customHeight="1" s="92"/>
+    <row r="679" ht="16.5" customHeight="1" s="92"/>
+    <row r="680" ht="16.5" customHeight="1" s="92"/>
+    <row r="681" ht="16.5" customHeight="1" s="92"/>
+    <row r="682" ht="16.5" customHeight="1" s="92"/>
+    <row r="683" ht="16.5" customHeight="1" s="92"/>
+    <row r="684" ht="16.5" customHeight="1" s="92"/>
+    <row r="685" ht="16.5" customHeight="1" s="92"/>
+    <row r="686" ht="16.5" customHeight="1" s="92"/>
+    <row r="687" ht="16.5" customHeight="1" s="92"/>
+    <row r="688" ht="16.5" customHeight="1" s="92"/>
+    <row r="689" ht="16.5" customHeight="1" s="92"/>
+    <row r="690" ht="16.5" customHeight="1" s="92"/>
+    <row r="691" ht="16.5" customHeight="1" s="92"/>
+    <row r="692" ht="16.5" customHeight="1" s="92"/>
+    <row r="693" ht="16.5" customHeight="1" s="92"/>
+    <row r="694" ht="16.5" customHeight="1" s="92"/>
+    <row r="695" ht="16.5" customHeight="1" s="92"/>
+    <row r="696" ht="16.5" customHeight="1" s="92"/>
+    <row r="697" ht="16.5" customHeight="1" s="92"/>
+    <row r="698" ht="16.5" customHeight="1" s="92"/>
+    <row r="699" ht="16.5" customHeight="1" s="92"/>
+    <row r="700" ht="16.5" customHeight="1" s="92"/>
+    <row r="701" ht="16.5" customHeight="1" s="92"/>
+    <row r="702" ht="16.5" customHeight="1" s="92"/>
+    <row r="703" ht="16.5" customHeight="1" s="92"/>
+    <row r="704" ht="16.5" customHeight="1" s="92"/>
+    <row r="705" ht="16.5" customHeight="1" s="92"/>
+    <row r="706" ht="16.5" customHeight="1" s="92"/>
+    <row r="707" ht="16.5" customHeight="1" s="92"/>
+    <row r="708" ht="16.5" customHeight="1" s="92"/>
+    <row r="709" ht="16.5" customHeight="1" s="92"/>
+    <row r="710" ht="16.5" customHeight="1" s="92"/>
+    <row r="711" ht="16.5" customHeight="1" s="92"/>
+    <row r="712" ht="16.5" customHeight="1" s="92"/>
+    <row r="713" ht="16.5" customHeight="1" s="92"/>
+    <row r="714" ht="16.5" customHeight="1" s="92"/>
+    <row r="715" ht="16.5" customHeight="1" s="92"/>
+    <row r="716" ht="16.5" customHeight="1" s="92"/>
+    <row r="717" ht="16.5" customHeight="1" s="92"/>
+    <row r="718" ht="16.5" customHeight="1" s="92"/>
+    <row r="719" ht="16.5" customHeight="1" s="92"/>
+    <row r="720" ht="16.5" customHeight="1" s="92"/>
+    <row r="721" ht="16.5" customHeight="1" s="92"/>
+    <row r="722" ht="16.5" customHeight="1" s="92"/>
+    <row r="723" ht="16.5" customHeight="1" s="92"/>
+    <row r="724" ht="16.5" customHeight="1" s="92"/>
+    <row r="725" ht="16.5" customHeight="1" s="92"/>
+    <row r="726" ht="16.5" customHeight="1" s="92"/>
+    <row r="727" ht="16.5" customHeight="1" s="92"/>
+    <row r="728" ht="16.5" customHeight="1" s="92"/>
+    <row r="729" ht="16.5" customHeight="1" s="92"/>
+    <row r="730" ht="16.5" customHeight="1" s="92"/>
+    <row r="731" ht="16.5" customHeight="1" s="92"/>
+    <row r="732" ht="16.5" customHeight="1" s="92"/>
+    <row r="733" ht="16.5" customHeight="1" s="92"/>
+    <row r="734" ht="16.5" customHeight="1" s="92"/>
+    <row r="735" ht="16.5" customHeight="1" s="92"/>
+    <row r="736" ht="16.5" customHeight="1" s="92"/>
+    <row r="737" ht="16.5" customHeight="1" s="92"/>
+    <row r="738" ht="16.5" customHeight="1" s="92"/>
+    <row r="739" ht="16.5" customHeight="1" s="92"/>
+    <row r="740" ht="16.5" customHeight="1" s="92"/>
+    <row r="741" ht="16.5" customHeight="1" s="92"/>
+    <row r="742" ht="16.5" customHeight="1" s="92"/>
+    <row r="743" ht="16.5" customHeight="1" s="92"/>
+    <row r="744" ht="16.5" customHeight="1" s="92"/>
+    <row r="745" ht="16.5" customHeight="1" s="92"/>
+    <row r="746" ht="16.5" customHeight="1" s="92"/>
+    <row r="747" ht="16.5" customHeight="1" s="92"/>
+    <row r="748" ht="16.5" customHeight="1" s="92"/>
+    <row r="749" ht="16.5" customHeight="1" s="92"/>
+    <row r="750" ht="16.5" customHeight="1" s="92"/>
+    <row r="751" ht="16.5" customHeight="1" s="92"/>
+    <row r="752" ht="16.5" customHeight="1" s="92"/>
+    <row r="753" ht="16.5" customHeight="1" s="92"/>
+    <row r="754" ht="16.5" customHeight="1" s="92"/>
+    <row r="755" ht="16.5" customHeight="1" s="92"/>
+    <row r="756" ht="16.5" customHeight="1" s="92"/>
+    <row r="757" ht="16.5" customHeight="1" s="92"/>
+    <row r="758" ht="16.5" customHeight="1" s="92"/>
+    <row r="759" ht="16.5" customHeight="1" s="92"/>
+    <row r="760" ht="16.5" customHeight="1" s="92"/>
+    <row r="761" ht="16.5" customHeight="1" s="92"/>
+    <row r="762" ht="16.5" customHeight="1" s="92"/>
+    <row r="763" ht="16.5" customHeight="1" s="92"/>
+    <row r="764" ht="16.5" customHeight="1" s="92"/>
+    <row r="765" ht="16.5" customHeight="1" s="92"/>
+    <row r="766" ht="16.5" customHeight="1" s="92"/>
+    <row r="767" ht="16.5" customHeight="1" s="92"/>
+    <row r="768" ht="16.5" customHeight="1" s="92"/>
+    <row r="769" ht="16.5" customHeight="1" s="92"/>
+    <row r="770" ht="16.5" customHeight="1" s="92"/>
+    <row r="771" ht="16.5" customHeight="1" s="92"/>
+    <row r="772" ht="16.5" customHeight="1" s="92"/>
+    <row r="773" ht="16.5" customHeight="1" s="92"/>
+    <row r="774" ht="16.5" customHeight="1" s="92"/>
+    <row r="775" ht="16.5" customHeight="1" s="92"/>
+    <row r="776" ht="16.5" customHeight="1" s="92"/>
+    <row r="777" ht="16.5" customHeight="1" s="92"/>
+    <row r="778" ht="16.5" customHeight="1" s="92"/>
+    <row r="779" ht="16.5" customHeight="1" s="92"/>
+    <row r="780" ht="16.5" customHeight="1" s="92"/>
+    <row r="781" ht="16.5" customHeight="1" s="92"/>
+    <row r="782" ht="16.5" customHeight="1" s="92"/>
+    <row r="783" ht="16.5" customHeight="1" s="92"/>
+    <row r="784" ht="16.5" customHeight="1" s="92"/>
+    <row r="785" ht="16.5" customHeight="1" s="92"/>
+    <row r="786" ht="16.5" customHeight="1" s="92"/>
+    <row r="787" ht="16.5" customHeight="1" s="92"/>
+    <row r="788" ht="16.5" customHeight="1" s="92"/>
+    <row r="789" ht="16.5" customHeight="1" s="92"/>
+    <row r="790" ht="16.5" customHeight="1" s="92"/>
+    <row r="791" ht="16.5" customHeight="1" s="92"/>
+    <row r="792" ht="16.5" customHeight="1" s="92"/>
+    <row r="793" ht="16.5" customHeight="1" s="92"/>
+    <row r="794" ht="16.5" customHeight="1" s="92"/>
+    <row r="795" ht="16.5" customHeight="1" s="92"/>
+    <row r="796" ht="16.5" customHeight="1" s="92"/>
+    <row r="797" ht="16.5" customHeight="1" s="92"/>
+    <row r="798" ht="16.5" customHeight="1" s="92"/>
+    <row r="799" ht="16.5" customHeight="1" s="92"/>
+    <row r="800" ht="16.5" customHeight="1" s="92"/>
+    <row r="801" ht="16.5" customHeight="1" s="92"/>
+    <row r="802" ht="16.5" customHeight="1" s="92"/>
+    <row r="803" ht="16.5" customHeight="1" s="92"/>
+    <row r="804" ht="16.5" customHeight="1" s="92"/>
+    <row r="805" ht="16.5" customHeight="1" s="92"/>
+    <row r="806" ht="16.5" customHeight="1" s="92"/>
+    <row r="807" ht="16.5" customHeight="1" s="92"/>
+    <row r="808" ht="16.5" customHeight="1" s="92"/>
+    <row r="809" ht="16.5" customHeight="1" s="92"/>
+    <row r="810" ht="16.5" customHeight="1" s="92"/>
+    <row r="811" ht="16.5" customHeight="1" s="92"/>
+    <row r="812" ht="16.5" customHeight="1" s="92"/>
+    <row r="813" ht="16.5" customHeight="1" s="92"/>
+    <row r="814" ht="16.5" customHeight="1" s="92"/>
+    <row r="815" ht="16.5" customHeight="1" s="92"/>
+    <row r="816" ht="16.5" customHeight="1" s="92"/>
+    <row r="817" ht="16.5" customHeight="1" s="92"/>
+    <row r="818" ht="16.5" customHeight="1" s="92"/>
+    <row r="819" ht="16.5" customHeight="1" s="92"/>
+    <row r="820" ht="16.5" customHeight="1" s="92"/>
+    <row r="821" ht="16.5" customHeight="1" s="92"/>
+    <row r="822" ht="16.5" customHeight="1" s="92"/>
+    <row r="823" ht="16.5" customHeight="1" s="92"/>
+    <row r="824" ht="16.5" customHeight="1" s="92"/>
+    <row r="825" ht="16.5" customHeight="1" s="92"/>
+    <row r="826" ht="16.5" customHeight="1" s="92"/>
+    <row r="827" ht="16.5" customHeight="1" s="92"/>
+    <row r="828" ht="16.5" customHeight="1" s="92"/>
+    <row r="829" ht="16.5" customHeight="1" s="92"/>
+    <row r="830" ht="16.5" customHeight="1" s="92"/>
+    <row r="831" ht="16.5" customHeight="1" s="92"/>
+    <row r="832" ht="16.5" customHeight="1" s="92"/>
+    <row r="833" ht="16.5" customHeight="1" s="92"/>
+    <row r="834" ht="16.5" customHeight="1" s="92"/>
+    <row r="835" ht="16.5" customHeight="1" s="92"/>
+    <row r="836" ht="16.5" customHeight="1" s="92"/>
+    <row r="837" ht="16.5" customHeight="1" s="92"/>
+    <row r="838" ht="16.5" customHeight="1" s="92"/>
+    <row r="839" ht="16.5" customHeight="1" s="92"/>
+    <row r="840" ht="16.5" customHeight="1" s="92"/>
+    <row r="841" ht="16.5" customHeight="1" s="92"/>
+    <row r="842" ht="16.5" customHeight="1" s="92"/>
+    <row r="843" ht="16.5" customHeight="1" s="92"/>
+    <row r="844" ht="16.5" customHeight="1" s="92"/>
+    <row r="845" ht="16.5" customHeight="1" s="92"/>
+    <row r="846" ht="16.5" customHeight="1" s="92"/>
+    <row r="847" ht="16.5" customHeight="1" s="92"/>
+    <row r="848" ht="16.5" customHeight="1" s="92"/>
+    <row r="849" ht="16.5" customHeight="1" s="92"/>
+    <row r="850" ht="16.5" customHeight="1" s="92"/>
+    <row r="851" ht="16.5" customHeight="1" s="92"/>
+    <row r="852" ht="16.5" customHeight="1" s="92"/>
+    <row r="853" ht="16.5" customHeight="1" s="92"/>
+    <row r="854" ht="16.5" customHeight="1" s="92"/>
+    <row r="855" ht="16.5" customHeight="1" s="92"/>
+    <row r="856" ht="16.5" customHeight="1" s="92"/>
+    <row r="857" ht="16.5" customHeight="1" s="92"/>
+    <row r="858" ht="16.5" customHeight="1" s="92"/>
+    <row r="859" ht="16.5" customHeight="1" s="92"/>
+    <row r="860" ht="16.5" customHeight="1" s="92"/>
+    <row r="861" ht="16.5" customHeight="1" s="92"/>
+    <row r="862" ht="16.5" customHeight="1" s="92"/>
+    <row r="863" ht="16.5" customHeight="1" s="92"/>
+    <row r="864" ht="16.5" customHeight="1" s="92"/>
+    <row r="865" ht="16.5" customHeight="1" s="92"/>
+    <row r="866" ht="16.5" customHeight="1" s="92"/>
+    <row r="867" ht="16.5" customHeight="1" s="92"/>
+    <row r="868" ht="16.5" customHeight="1" s="92"/>
+    <row r="869" ht="16.5" customHeight="1" s="92"/>
+    <row r="870" ht="16.5" customHeight="1" s="92"/>
+    <row r="871" ht="16.5" customHeight="1" s="92"/>
+    <row r="872" ht="16.5" customHeight="1" s="92"/>
+    <row r="873" ht="16.5" customHeight="1" s="92"/>
+    <row r="874" ht="16.5" customHeight="1" s="92"/>
+    <row r="875" ht="16.5" customHeight="1" s="92"/>
+    <row r="876" ht="16.5" customHeight="1" s="92"/>
+    <row r="877" ht="16.5" customHeight="1" s="92"/>
+    <row r="878" ht="16.5" customHeight="1" s="92"/>
+    <row r="879" ht="16.5" customHeight="1" s="92"/>
+    <row r="880" ht="16.5" customHeight="1" s="92"/>
+    <row r="881" ht="16.5" customHeight="1" s="92"/>
+    <row r="882" ht="16.5" customHeight="1" s="92"/>
+    <row r="883" ht="16.5" customHeight="1" s="92"/>
+    <row r="884" ht="16.5" customHeight="1" s="92"/>
+    <row r="885" ht="16.5" customHeight="1" s="92"/>
+    <row r="886" ht="16.5" customHeight="1" s="92"/>
+    <row r="887" ht="16.5" customHeight="1" s="92"/>
+    <row r="888" ht="16.5" customHeight="1" s="92"/>
+    <row r="889" ht="16.5" customHeight="1" s="92"/>
+    <row r="890" ht="16.5" customHeight="1" s="92"/>
+    <row r="891" ht="16.5" customHeight="1" s="92"/>
+    <row r="892" ht="16.5" customHeight="1" s="92"/>
+    <row r="893" ht="16.5" customHeight="1" s="92"/>
+    <row r="894" ht="16.5" customHeight="1" s="92"/>
+    <row r="895" ht="16.5" customHeight="1" s="92"/>
+    <row r="896" ht="16.5" customHeight="1" s="92"/>
+    <row r="897" ht="16.5" customHeight="1" s="92"/>
+    <row r="898" ht="16.5" customHeight="1" s="92"/>
+    <row r="899" ht="16.5" customHeight="1" s="92"/>
+    <row r="900" ht="16.5" customHeight="1" s="92"/>
+    <row r="901" ht="16.5" customHeight="1" s="92"/>
+    <row r="902" ht="16.5" customHeight="1" s="92"/>
+    <row r="903" ht="16.5" customHeight="1" s="92"/>
+    <row r="904" ht="16.5" customHeight="1" s="92"/>
+    <row r="905" ht="16.5" customHeight="1" s="92"/>
+    <row r="906" ht="16.5" customHeight="1" s="92"/>
+    <row r="907" ht="16.5" customHeight="1" s="92"/>
+    <row r="908" ht="16.5" customHeight="1" s="92"/>
+    <row r="909" ht="16.5" customHeight="1" s="92"/>
+    <row r="910" ht="16.5" customHeight="1" s="92"/>
+    <row r="911" ht="16.5" customHeight="1" s="92"/>
+    <row r="912" ht="16.5" customHeight="1" s="92"/>
+    <row r="913" ht="16.5" customHeight="1" s="92"/>
+    <row r="914" ht="16.5" customHeight="1" s="92"/>
+    <row r="915" ht="16.5" customHeight="1" s="92"/>
+    <row r="916" ht="16.5" customHeight="1" s="92"/>
+    <row r="917" ht="16.5" customHeight="1" s="92"/>
+    <row r="918" ht="16.5" customHeight="1" s="92"/>
+    <row r="919" ht="16.5" customHeight="1" s="92"/>
+    <row r="920" ht="16.5" customHeight="1" s="92"/>
+    <row r="921" ht="16.5" customHeight="1" s="92"/>
+    <row r="922" ht="16.5" customHeight="1" s="92"/>
+    <row r="923" ht="16.5" customHeight="1" s="92"/>
+    <row r="924" ht="16.5" customHeight="1" s="92"/>
+    <row r="925" ht="16.5" customHeight="1" s="92"/>
+    <row r="926" ht="16.5" customHeight="1" s="92"/>
+    <row r="927" ht="16.5" customHeight="1" s="92"/>
+    <row r="928" ht="16.5" customHeight="1" s="92"/>
+    <row r="929" ht="16.5" customHeight="1" s="92"/>
+    <row r="930" ht="16.5" customHeight="1" s="92"/>
+    <row r="931" ht="16.5" customHeight="1" s="92"/>
+    <row r="932" ht="16.5" customHeight="1" s="92"/>
+    <row r="933" ht="16.5" customHeight="1" s="92"/>
+    <row r="934" ht="16.5" customHeight="1" s="92"/>
+    <row r="935" ht="16.5" customHeight="1" s="92"/>
+    <row r="936" ht="16.5" customHeight="1" s="92"/>
+    <row r="937" ht="16.5" customHeight="1" s="92"/>
+    <row r="938" ht="16.5" customHeight="1" s="92"/>
+    <row r="939" ht="16.5" customHeight="1" s="92"/>
+    <row r="940" ht="16.5" customHeight="1" s="92"/>
+    <row r="941" ht="16.5" customHeight="1" s="92"/>
+    <row r="942" ht="16.5" customHeight="1" s="92"/>
+    <row r="943" ht="16.5" customHeight="1" s="92"/>
+    <row r="944" ht="16.5" customHeight="1" s="92"/>
+    <row r="945" ht="16.5" customHeight="1" s="92"/>
+    <row r="946" ht="16.5" customHeight="1" s="92"/>
+    <row r="947" ht="16.5" customHeight="1" s="92"/>
+    <row r="948" ht="16.5" customHeight="1" s="92"/>
+    <row r="949" ht="16.5" customHeight="1" s="92"/>
+    <row r="950" ht="16.5" customHeight="1" s="92"/>
+    <row r="951" ht="16.5" customHeight="1" s="92"/>
+    <row r="952" ht="16.5" customHeight="1" s="92"/>
+    <row r="953" ht="16.5" customHeight="1" s="92"/>
+    <row r="954" ht="16.5" customHeight="1" s="92"/>
+    <row r="955" ht="16.5" customHeight="1" s="92"/>
+    <row r="956" ht="16.5" customHeight="1" s="92"/>
+    <row r="957" ht="16.5" customHeight="1" s="92"/>
+    <row r="958" ht="16.5" customHeight="1" s="92"/>
+    <row r="959" ht="16.5" customHeight="1" s="92"/>
+    <row r="960" ht="16.5" customHeight="1" s="92"/>
+    <row r="961" ht="16.5" customHeight="1" s="92"/>
+    <row r="962" ht="16.5" customHeight="1" s="92"/>
+    <row r="963" ht="16.5" customHeight="1" s="92"/>
+    <row r="964" ht="16.5" customHeight="1" s="92"/>
+    <row r="965" ht="16.5" customHeight="1" s="92"/>
+    <row r="966" ht="16.5" customHeight="1" s="92"/>
+    <row r="967" ht="16.5" customHeight="1" s="92"/>
+    <row r="968" ht="16.5" customHeight="1" s="92"/>
+    <row r="969" ht="16.5" customHeight="1" s="92"/>
+    <row r="970" ht="16.5" customHeight="1" s="92"/>
+    <row r="971" ht="16.5" customHeight="1" s="92"/>
+    <row r="972" ht="16.5" customHeight="1" s="92"/>
+    <row r="973" ht="16.5" customHeight="1" s="92"/>
+    <row r="974" ht="16.5" customHeight="1" s="92"/>
+    <row r="975" ht="16.5" customHeight="1" s="92"/>
+    <row r="976" ht="16.5" customHeight="1" s="92"/>
+    <row r="977" ht="16.5" customHeight="1" s="92"/>
+    <row r="978" ht="16.5" customHeight="1" s="92"/>
+    <row r="979" ht="16.5" customHeight="1" s="92"/>
+    <row r="980" ht="16.5" customHeight="1" s="92"/>
+    <row r="981" ht="16.5" customHeight="1" s="92"/>
+    <row r="982" ht="16.5" customHeight="1" s="92"/>
+    <row r="983" ht="16.5" customHeight="1" s="92"/>
+    <row r="984" ht="16.5" customHeight="1" s="92"/>
+    <row r="985" ht="16.5" customHeight="1" s="92"/>
+    <row r="986" ht="16.5" customHeight="1" s="92"/>
+    <row r="987" ht="16.5" customHeight="1" s="92"/>
+    <row r="988" ht="16.5" customHeight="1" s="92"/>
+    <row r="989" ht="16.5" customHeight="1" s="92"/>
+    <row r="990" ht="16.5" customHeight="1" s="92"/>
+    <row r="991" ht="16.5" customHeight="1" s="92"/>
+    <row r="992" ht="16.5" customHeight="1" s="92"/>
+    <row r="993" ht="16.5" customHeight="1" s="92"/>
+    <row r="994" ht="16.5" customHeight="1" s="92"/>
+    <row r="995" ht="16.5" customHeight="1" s="92"/>
+    <row r="996" ht="16.5" customHeight="1" s="92"/>
+    <row r="997" ht="16.5" customHeight="1" s="92"/>
+    <row r="998" ht="16.5" customHeight="1" s="92"/>
+    <row r="999" ht="16.5" customHeight="1" s="92"/>
+    <row r="1000" ht="16.5" customHeight="1" s="92"/>
+    <row r="1001" ht="16.5" customHeight="1" s="92"/>
+    <row r="1002" ht="16.5" customHeight="1" s="92"/>
+    <row r="1003" ht="16.5" customHeight="1" s="92"/>
+    <row r="1004" ht="16.5" customHeight="1" s="92"/>
+    <row r="1005" ht="16.5" customHeight="1" s="92"/>
+    <row r="1006" ht="16.5" customHeight="1" s="92"/>
+    <row r="1007" ht="16.5" customHeight="1" s="92"/>
+    <row r="1008" ht="16.5" customHeight="1" s="92"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>